<commit_message>
Dossier v3 : alignement sur le certificat Qualiopi, la base Airtable et la charte YEBA
- Coordonnées, assurance Hiscox, TVA (art. 293 B), mention EI, Qualiopi
  4 catégories valable jusqu'au 16/02/2029 et audit de surveillance planifié.
- Charte YEBA-IDENT-2026 : texte bleu ou noir, or réservé aux filets,
  interligne 1,3, bloc-marque et mention de transparence IA sur chaque document.
- Documents stagiaires recentrés sur les parcours certifiants en complément
  du socle officiel (avenant RI-06, conditions particulières CP-05,
  aménagements d'examen) ; doublons retirés ; règle cyclonique alignée.
- SOC-04 : socle documentaire et écarts relevés dans Airtable ; plan
  d'actions complété (médiateur, attestation 3511-SD, assurance IA, audit).
- Instantané des documents officiels Airtable dans sources/.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JZ6CWNerPeDJEuR1MPsUp5
</commit_message>
<xml_diff>
--- a/dossier-conformite-2026/livrables/05_Pilotage_annuel/PIL-03_Budget_tresorerie_tableau_de_bord.xlsx
+++ b/dossier-conformite-2026/livrables/05_Pilotage_annuel/PIL-03_Budget_tresorerie_tableau_de_bord.xlsx
@@ -29,7 +29,7 @@
     <numFmt numFmtId="167" formatCode="#,##0.00 &quot;€&quot;"/>
     <numFmt numFmtId="168" formatCode="mmmm yyyy"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +56,12 @@
     <font>
       <name val="Arial"/>
       <i val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="001B3A6B"/>
       <sz val="11"/>
     </font>
     <font>
@@ -114,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -127,6 +133,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -139,13 +146,13 @@
     <xf numFmtId="166" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -525,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -590,7 +597,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Vérifier le périmètre et la date d'audit de surveillance du certificat Qualiopi 25FOR02027.1</t>
+          <t>Corriger dans Airtable les écarts listés dans SOC-04 (catégories et validité Qualiopi, TVA, assurance, mention EI)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr"/>
@@ -602,12 +609,12 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Référentiels</t>
+          <t>Assurance</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Obtenir le REAC et le référentiel d'évaluation RPMS millésime 08 (DEETS ou ministère du Travail)</t>
+          <t>Faire confirmer par écrit au courtier ELASSUR que le module IA et le conseil sont couverts (exclusion « intelligence artificielle »)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr"/>
@@ -615,16 +622,16 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46346</v>
+        <v>46339</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Examen</t>
+          <t>Référentiels</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Décider : agrément de centre d'examen ou partenariat avec un centre agréé (document AGR-03)</t>
+          <t>Obtenir le REAC et le référentiel d'évaluation RPMS millésime 08 (DEETS ou ministère du Travail)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr"/>
@@ -632,16 +639,16 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46353</v>
+        <v>46346</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Locaux</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Réserver au Secrétariat Center les journées de la promotion MEM ; vérifier accessibilité, sanitaires, salle de pause</t>
+          <t>Décider : agrément de centre d'examen ou partenariat avec un centre agréé (document AGR-03)</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr"/>
@@ -649,16 +656,16 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46356</v>
+        <v>46353</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Sécurité</t>
+          <t>Fiscalité</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Plan de continuité cyclonique : contacts, formation à distance, procédure d'information des stagiaires</t>
+          <t>Avec l'expert-comptable : seuil de franchise de TVA applicable à La Réunion et demande de l'attestation 3511-SD avant les premières recettes des parcours</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr"/>
@@ -666,16 +673,16 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46357</v>
+        <v>46353</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Offre</t>
+          <t>Locaux</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>MEM — Promotion 1 : publier l'offre (Carif-Oref Réunion, KAIROS, Mon Compte Formation, site) ; informer Missions Locales et agences France Travail</t>
+          <t>Réserver au Secrétariat Center les 80 journées de la promotion MEM (100 € par jour)</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr"/>
@@ -683,16 +690,16 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46391</v>
+        <v>46356</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Partenaires</t>
+          <t>Sécurité</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>MEM — Promotion 1 : constituer le vivier d'entreprises d'accueil pour les périodes en entreprise</t>
+          <t>Plan de continuité cyclonique : contacts, formation à distance, procédure d'information des stagiaires</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr"/>
@@ -700,16 +707,16 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46391</v>
+        <v>46357</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Recrutement</t>
+          <t>Offre</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>MEM — Promotion 1 : 1re information collective</t>
+          <t>MEM — Promotion 1 : publier l'offre (Carif-Oref Réunion, KAIROS, Mon Compte Formation, site) ; informer Missions Locales et agences France Travail</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr"/>
@@ -717,16 +724,16 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46412</v>
+        <v>46367</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Examen</t>
+          <t>Juridique</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>MEM — Promotion 1 : déposer la demande d'agrément de session (démarche en ligne DEETS 974) ou signer la convention avec le centre agréé</t>
+          <t>Désigner un médiateur de la consommation (obligatoire avant tout contrat avec un particulier)</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr"/>
@@ -734,16 +741,16 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46419</v>
+        <v>46391</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>IA Act</t>
+          <t>Partenaires</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Former l'équipe à la maîtrise de l'IA (article 4) et faire signer la charte IA</t>
+          <t>MEM — Promotion 1 : constituer le vivier d'entreprises d'accueil pour les périodes en entreprise</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr"/>
@@ -751,7 +758,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46419</v>
+        <v>46391</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -760,7 +767,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>MEM — Promotion 1 : 2e information collective, entretiens, décisions d'admission, accords de financement</t>
+          <t>MEM — Promotion 1 : 1re information collective</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
@@ -768,16 +775,16 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46433</v>
+        <v>46402</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Administratif</t>
+          <t>Handicap</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>MEM — Promotion 1 : envoyer convocations, livret d'accueil, règlement intérieur, programme</t>
+          <t>Formaliser une convention ou un contact référencé avec l'Agefiph Océan Indien ou la Ressource Handicap Formation</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr"/>
@@ -785,16 +792,16 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46447</v>
+        <v>46412</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Formation</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>MEM — Promotion 1 : démarrage — attestations d'entrée, déclarations d'entrée sur les plateformes des financeurs</t>
+          <t>MEM — Promotion 1 : déposer la demande d'agrément de session (démarche en ligne DEETS 974) ou signer la convention avec le centre agréé</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr"/>
@@ -802,16 +809,16 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46450</v>
+        <v>46419</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Formation</t>
+          <t>IA Act</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>MEM — Promotion 1 : élection des délégués des stagiaires (entre la 20e et la 40e heure)</t>
+          <t>Former l'équipe à la maîtrise de l'IA (article 4) et faire signer la charte IA</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr"/>
@@ -819,16 +826,16 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46477</v>
+        <v>46419</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Obligation</t>
+          <t>Recrutement</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Renouveler l'attestation de vigilance URSSAF (tous les 6 mois)</t>
+          <t>MEM — Promotion 1 : 2e information collective, entretiens, décisions d'admission, accords de financement</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr"/>
@@ -836,16 +843,16 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46505</v>
+        <v>46430</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Entreprise</t>
+          <t>Locaux</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>MEM — Promotion 1 : conventions de la période en entreprise n° 1 signées</t>
+          <t>Remplir la fiche site tiers YEBA-DOC-15 pour le Secrétariat Center (sécurité, évacuation, accessibilité)</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr"/>
@@ -853,16 +860,16 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46507</v>
+        <v>46433</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>RGPD</t>
+          <t>Administratif</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Revue annuelle du registre des traitements et purge des données échues</t>
+          <t>MEM — Promotion 1 : envoyer convocations, livret d'accueil, règlement intérieur, programme</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr"/>
@@ -870,16 +877,16 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46533</v>
+        <v>46447</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Entreprise</t>
+          <t>Formation</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>MEM — Promotion 1 : appel ou visite des tuteurs (période n° 1)</t>
+          <t>MEM — Promotion 1 : démarrage — attestations d'entrée, déclarations d'entrée sur les plateformes des financeurs</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr"/>
@@ -887,16 +894,16 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46538</v>
+        <v>46450</v>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Obligation</t>
+          <t>Formation</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Déposer le bilan pédagogique et financier de 2026 (Mon Activité Formation)</t>
+          <t>MEM — Promotion 1 : élection des délégués des stagiaires (entre la 20e et la 40e heure)</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr"/>
@@ -904,16 +911,16 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46545</v>
+        <v>46461</v>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Offre</t>
+          <t>Qualité</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>RPMS — Promotion 1 : publier l'offre (Carif-Oref Réunion, KAIROS, Mon Compte Formation, site) ; informer Missions Locales et agences France Travail</t>
+          <t>Préparer l'audit de surveillance Qualiopi (fenêtre du 17/04/2027 au 17/12/2027) : matrice QUA-02, preuves de la promotion MEM</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr"/>
@@ -921,16 +928,16 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46569</v>
+        <v>46477</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Entreprise</t>
+          <t>Obligation</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>MEM — Promotion 1 : conventions de la période en entreprise n° 2 signées</t>
+          <t>Renouveler l'attestation de vigilance URSSAF (tous les 6 mois)</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr"/>
@@ -938,16 +945,16 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46574</v>
+        <v>46505</v>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Partenaires</t>
+          <t>Entreprise</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>RPMS — Promotion 1 : constituer le vivier d'entreprises d'accueil pour les périodes en entreprise</t>
+          <t>MEM — Promotion 1 : conventions de la période en entreprise n° 1 signées</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr"/>
@@ -955,16 +962,16 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46574</v>
+        <v>46507</v>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Recrutement</t>
+          <t>RGPD</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>RPMS — Promotion 1 : 1re information collective</t>
+          <t>Revue annuelle du registre des traitements et purge des données échues</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr"/>
@@ -972,7 +979,7 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46596</v>
+        <v>46533</v>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
@@ -981,7 +988,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>MEM — Promotion 1 : appel ou visite des tuteurs (période n° 2)</t>
+          <t>MEM — Promotion 1 : appel ou visite des tuteurs (période n° 1)</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr"/>
@@ -989,16 +996,16 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46605</v>
+        <v>46538</v>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Examen</t>
+          <t>Obligation</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>RPMS — Promotion 1 : déposer la demande d'agrément de session (démarche en ligne DEETS 974) ou signer la convention avec le centre agréé</t>
+          <t>Déposer le bilan pédagogique et financier de 2026 (Mon Activité Formation)</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr"/>
@@ -1006,16 +1013,16 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46605</v>
+        <v>46545</v>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Recrutement</t>
+          <t>Offre</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>RPMS — Promotion 1 : 2e information collective, entretiens, décisions d'admission, accords de financement</t>
+          <t>RPMS — Promotion 1 : publier l'offre (Carif-Oref Réunion, KAIROS, Mon Compte Formation, site) ; informer Missions Locales et agences France Travail</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr"/>
@@ -1023,16 +1030,16 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46608</v>
+        <v>46569</v>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Examen</t>
+          <t>Entreprise</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>MEM — Promotion 1 : dossiers professionnels, productions et attestations de période en entreprise complets</t>
+          <t>MEM — Promotion 1 : conventions de la période en entreprise n° 2 signées</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr"/>
@@ -1040,16 +1047,16 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46618</v>
+        <v>46574</v>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Administratif</t>
+          <t>Partenaires</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>MEM — Promotion 1 : évaluation à chaud, attestations de fin de formation, certificats de réalisation, facturation</t>
+          <t>RPMS — Promotion 1 : constituer le vivier d'entreprises d'accueil pour les périodes en entreprise</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr"/>
@@ -1057,16 +1064,16 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46622</v>
+        <v>46574</v>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Administratif</t>
+          <t>Recrutement</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>RPMS — Promotion 1 : envoyer convocations, livret d'accueil, règlement intérieur, programme</t>
+          <t>RPMS — Promotion 1 : 1re information collective</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr"/>
@@ -1074,16 +1081,16 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46622</v>
+        <v>46577</v>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Examen</t>
+          <t>Assurance</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>MEM — Promotion 1 : session de validation [À VÉRIFIER : date confirmée]</t>
+          <t>Décider du renouvellement de la RC Pro Hiscox (échéance 10/09/2027, préavis de 2 mois)</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr"/>
@@ -1091,16 +1098,16 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46636</v>
+        <v>46596</v>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Formation</t>
+          <t>Entreprise</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>RPMS — Promotion 1 : démarrage — attestations d'entrée, déclarations d'entrée sur les plateformes des financeurs</t>
+          <t>MEM — Promotion 1 : appel ou visite des tuteurs (période n° 2)</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr"/>
@@ -1108,16 +1115,16 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46639</v>
+        <v>46605</v>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Formation</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>RPMS — Promotion 1 : élection des délégués des stagiaires (entre la 20e et la 40e heure)</t>
+          <t>RPMS — Promotion 1 : déposer la demande d'agrément de session (démarche en ligne DEETS 974) ou signer la convention avec le centre agréé</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr"/>
@@ -1125,16 +1132,16 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46660</v>
+        <v>46605</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Obligation</t>
+          <t>Recrutement</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Renouveler l'attestation de vigilance URSSAF (tous les 6 mois)</t>
+          <t>RPMS — Promotion 1 : 2e information collective, entretiens, décisions d'admission, accords de financement</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr"/>
@@ -1142,16 +1149,16 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46687</v>
+        <v>46608</v>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Entreprise</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>RPMS — Promotion 1 : conventions de la période en entreprise n° 1 signées</t>
+          <t>MEM — Promotion 1 : dossiers professionnels, productions et attestations de période en entreprise complets</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr"/>
@@ -1159,16 +1166,16 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46709</v>
+        <v>46618</v>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Qualité</t>
+          <t>Administratif</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>MEM — Promotion 1 : questionnaire à froid (3 mois)</t>
+          <t>MEM — Promotion 1 : évaluation à chaud, attestations de fin de formation, certificats de réalisation, facturation</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr"/>
@@ -1176,16 +1183,16 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46713</v>
+        <v>46622</v>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Entreprise</t>
+          <t>Administratif</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>RPMS — Promotion 1 : appel ou visite des tuteurs (période n° 1)</t>
+          <t>RPMS — Promotion 1 : envoyer convocations, livret d'accueil, règlement intérieur, programme</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr"/>
@@ -1193,16 +1200,16 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46771</v>
+        <v>46622</v>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Entreprise</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>RPMS — Promotion 1 : conventions de la période en entreprise n° 2 signées</t>
+          <t>MEM — Promotion 1 : session de validation [À VÉRIFIER : date confirmée]</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr"/>
@@ -1210,16 +1217,16 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46797</v>
+        <v>46636</v>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Entreprise</t>
+          <t>Formation</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>RPMS — Promotion 1 : appel ou visite des tuteurs (période n° 2)</t>
+          <t>RPMS — Promotion 1 : démarrage — attestations d'entrée, déclarations d'entrée sur les plateformes des financeurs</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr"/>
@@ -1227,16 +1234,16 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46800</v>
+        <v>46639</v>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Qualité</t>
+          <t>Formation</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>MEM — Promotion 1 : enquête d'insertion à 6 mois et mise à jour des résultats publiés</t>
+          <t>RPMS — Promotion 1 : élection des délégués des stagiaires (entre la 20e et la 40e heure)</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr"/>
@@ -1244,16 +1251,16 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46804</v>
+        <v>46660</v>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Examen</t>
+          <t>Obligation</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>RPMS — Promotion 1 : dossiers professionnels, productions et attestations de période en entreprise complets</t>
+          <t>Renouveler l'attestation de vigilance URSSAF (tous les 6 mois)</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr"/>
@@ -1261,16 +1268,16 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46812</v>
+        <v>46687</v>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Administratif</t>
+          <t>Entreprise</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>RPMS — Promotion 1 : évaluation à chaud, attestations de fin de formation, certificats de réalisation, facturation</t>
+          <t>RPMS — Promotion 1 : conventions de la période en entreprise n° 1 signées</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr"/>
@@ -1278,16 +1285,16 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46818</v>
+        <v>46709</v>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Examen</t>
+          <t>Qualité</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>RPMS — Promotion 1 : session de validation [À VÉRIFIER : date confirmée]</t>
+          <t>MEM — Promotion 1 : questionnaire à froid (3 mois)</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr"/>
@@ -1295,16 +1302,16 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46843</v>
+        <v>46713</v>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Obligation</t>
+          <t>Entreprise</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Renouveler l'attestation de vigilance URSSAF (tous les 6 mois)</t>
+          <t>RPMS — Promotion 1 : appel ou visite des tuteurs (période n° 1)</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr"/>
@@ -1312,16 +1319,16 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46875</v>
+        <v>46771</v>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>RGPD</t>
+          <t>Entreprise</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Revue annuelle du registre des traitements et purge des données échues</t>
+          <t>RPMS — Promotion 1 : conventions de la période en entreprise n° 2 signées</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr"/>
@@ -1329,16 +1336,16 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46903</v>
+        <v>46797</v>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Qualité</t>
+          <t>Entreprise</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>RPMS — Promotion 1 : questionnaire à froid (3 mois)</t>
+          <t>RPMS — Promotion 1 : appel ou visite des tuteurs (période n° 2)</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr"/>
@@ -1346,16 +1353,16 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46904</v>
+        <v>46800</v>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Obligation</t>
+          <t>Qualité</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Déposer le bilan pédagogique et financier de 2027 (Mon Activité Formation)</t>
+          <t>MEM — Promotion 1 : enquête d'insertion à 6 mois et mise à jour des résultats publiés</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr"/>
@@ -1363,16 +1370,16 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46994</v>
+        <v>46804</v>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Qualité</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>RPMS — Promotion 1 : enquête d'insertion à 6 mois et mise à jour des résultats publiés</t>
+          <t>RPMS — Promotion 1 : dossiers professionnels, productions et attestations de période en entreprise complets</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr"/>
@@ -1380,20 +1387,139 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>47028</v>
+        <v>46812</v>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Obligation</t>
+          <t>Administratif</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Renouveler l'attestation de vigilance URSSAF (tous les 6 mois)</t>
+          <t>RPMS — Promotion 1 : évaluation à chaud, attestations de fin de formation, certificats de réalisation, facturation</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr"/>
       <c r="E50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46818</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>RPMS — Promotion 1 : session de validation [À VÉRIFIER : date confirmée]</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr"/>
+      <c r="E51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46843</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Obligation</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Renouveler l'attestation de vigilance URSSAF (tous les 6 mois)</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr"/>
+      <c r="E52" s="3" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46875</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>RGPD</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Revue annuelle du registre des traitements et purge des données échues</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr"/>
+      <c r="E53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46903</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Qualité</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>RPMS — Promotion 1 : questionnaire à froid (3 mois)</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr"/>
+      <c r="E54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46904</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Obligation</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Déposer le bilan pédagogique et financier de 2027 (Mon Activité Formation)</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr"/>
+      <c r="E55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46994</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Qualité</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>RPMS — Promotion 1 : enquête d'insertion à 6 mois et mise à jour des résultats publiés</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr"/>
+      <c r="E56" s="3" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>47028</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Obligation</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Renouveler l'attestation de vigilance URSSAF (tous les 6 mois)</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr"/>
+      <c r="E57" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1435,6 +1561,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>TVA : franchise en base (art. 293 B du CGI). Si le chiffre d'affaires annuel dépasse le seuil de franchise, la formation reste sans TVA uniquement avec l'attestation 3511-SD — à voir avec l'expert-comptable.</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -1458,7 +1591,7 @@
           <t>Nombre de stagiaires</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="7" t="n">
         <v>10</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -1473,7 +1606,7 @@
           <t>Prix du parcours par stagiaire</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n"/>
+      <c r="B6" s="8" t="n"/>
       <c r="C6" s="3" t="inlineStr">
         <is>
           <t>[À COMPLÉTER] — prix de vente, net de TVA</t>
@@ -1486,7 +1619,7 @@
           <t>Heures en centre</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="9" t="n">
         <v>560</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -1501,7 +1634,7 @@
           <t>Journées en centre</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="9" t="n">
         <v>80</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -1516,7 +1649,7 @@
           <t>Location de salle par jour</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="8" t="n">
         <v>100</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -1531,7 +1664,7 @@
           <t>Heures assurées par des formateurs externes</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="7" t="n">
         <v>0</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1546,7 +1679,7 @@
           <t>Coût horaire d'un formateur externe</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n"/>
+      <c r="B11" s="8" t="n"/>
       <c r="C11" s="3" t="inlineStr">
         <is>
           <t>[À COMPLÉTER]</t>
@@ -1559,7 +1692,7 @@
           <t>Ordinateurs portables (achat ou location)</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n"/>
+      <c r="B12" s="8" t="n"/>
       <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Indispensables pour T2 et l'épreuve de mise en situation du MEM</t>
@@ -1572,7 +1705,7 @@
           <t>Coût d'examen par candidat (centre agréé partenaire)</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n"/>
+      <c r="B13" s="8" t="n"/>
       <c r="C13" s="3" t="inlineStr">
         <is>
           <t>[À COMPLÉTER] si pas d'agrément propre</t>
@@ -1585,7 +1718,7 @@
           <t>Jury blanc (défraiement)</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n"/>
+      <c r="B14" s="8" t="n"/>
       <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Professionnels invités</t>
@@ -1598,7 +1731,7 @@
           <t>Communication et recrutement</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n"/>
+      <c r="B15" s="8" t="n"/>
       <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Informations collectives, supports</t>
@@ -1611,7 +1744,7 @@
           <t>Assurances, logiciels, frais administratifs</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n"/>
+      <c r="B16" s="8" t="n"/>
       <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Quote-part de la promotion</t>
@@ -1641,7 +1774,7 @@
           <t>Chiffre d'affaires</t>
         </is>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="10">
         <f>B5*B6</f>
         <v/>
       </c>
@@ -1657,7 +1790,7 @@
           <t>Location de salle</t>
         </is>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="10">
         <f>B8*B9</f>
         <v/>
       </c>
@@ -1673,7 +1806,7 @@
           <t>Formateurs externes</t>
         </is>
       </c>
-      <c r="B21" s="9">
+      <c r="B21" s="10">
         <f>B10*B11</f>
         <v/>
       </c>
@@ -1689,7 +1822,7 @@
           <t>Matériel informatique</t>
         </is>
       </c>
-      <c r="B22" s="9">
+      <c r="B22" s="10">
         <f>B12</f>
         <v/>
       </c>
@@ -1701,7 +1834,7 @@
           <t>Examens</t>
         </is>
       </c>
-      <c r="B23" s="9">
+      <c r="B23" s="10">
         <f>B5*B13</f>
         <v/>
       </c>
@@ -1717,7 +1850,7 @@
           <t>Jury blanc</t>
         </is>
       </c>
-      <c r="B24" s="9">
+      <c r="B24" s="10">
         <f>B14</f>
         <v/>
       </c>
@@ -1729,7 +1862,7 @@
           <t>Communication</t>
         </is>
       </c>
-      <c r="B25" s="9">
+      <c r="B25" s="10">
         <f>B15</f>
         <v/>
       </c>
@@ -1741,31 +1874,31 @@
           <t>Frais généraux</t>
         </is>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="10">
         <f>B16</f>
         <v/>
       </c>
       <c r="C26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>Total des charges</t>
         </is>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="10">
         <f>SUM(B20:B26)</f>
         <v/>
       </c>
       <c r="C27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="inlineStr">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>Résultat de la promotion</t>
         </is>
       </c>
-      <c r="B28" s="9">
+      <c r="B28" s="10">
         <f>B19-B27</f>
         <v/>
       </c>
@@ -1776,12 +1909,12 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="inlineStr">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Seuil de rentabilité (stagiaires)</t>
         </is>
       </c>
-      <c r="B29" s="8">
+      <c r="B29" s="9">
         <f>IF(B6&gt;0,ROUNDUP((B27-B5*B13)/(B6-B13),0),"")</f>
         <v/>
       </c>
@@ -1797,7 +1930,7 @@
           <t>Coût de la salle par heure-stagiaire</t>
         </is>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="12">
         <f>IF(B5&gt;0,B20/(B7*B5),"")</f>
         <v/>
       </c>
@@ -1843,36 +1976,36 @@
           <t>Solde cumulé</t>
         </is>
       </c>
-      <c r="I33" s="12" t="inlineStr">
+      <c r="I33" s="13" t="inlineStr">
         <is>
           <t>Échéancier d'encaissement</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="n">
+      <c r="A34" s="14" t="n">
         <v>46447</v>
       </c>
-      <c r="B34" s="14" t="n">
+      <c r="B34" s="15" t="n">
         <v>22</v>
       </c>
-      <c r="C34" s="9">
+      <c r="C34" s="10">
         <f>IF(0=0+$J$37,$B$19*$J$34,0)+IF(0=3+$J$37,$B$19*$J$35,0)+IF(0=5+$J$37,$B$19*$J$36,0)</f>
         <v/>
       </c>
-      <c r="D34" s="9">
+      <c r="D34" s="10">
         <f>-B34*$B$9</f>
         <v/>
       </c>
-      <c r="E34" s="9">
+      <c r="E34" s="10">
         <f>-($B$21+$B$22+$B$23+$B$24+$B$25+$B$26)/6</f>
         <v/>
       </c>
-      <c r="F34" s="9">
+      <c r="F34" s="10">
         <f>C34+D34+E34</f>
         <v/>
       </c>
-      <c r="G34" s="9">
+      <c r="G34" s="10">
         <f>F34</f>
         <v/>
       </c>
@@ -1881,34 +2014,34 @@
           <t>À l'entrée</t>
         </is>
       </c>
-      <c r="J34" s="15" t="n">
+      <c r="J34" s="16" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="n">
+      <c r="A35" s="14" t="n">
         <v>46478</v>
       </c>
-      <c r="B35" s="14" t="n">
+      <c r="B35" s="15" t="n">
         <v>22</v>
       </c>
-      <c r="C35" s="9">
+      <c r="C35" s="10">
         <f>IF(1=0+$J$37,$B$19*$J$34,0)+IF(1=3+$J$37,$B$19*$J$35,0)+IF(1=5+$J$37,$B$19*$J$36,0)</f>
         <v/>
       </c>
-      <c r="D35" s="9">
+      <c r="D35" s="10">
         <f>-B35*$B$9</f>
         <v/>
       </c>
-      <c r="E35" s="9">
+      <c r="E35" s="10">
         <f>-($B$21+$B$22+$B$23+$B$24+$B$25+$B$26)/6</f>
         <v/>
       </c>
-      <c r="F35" s="9">
+      <c r="F35" s="10">
         <f>C35+D35+E35</f>
         <v/>
       </c>
-      <c r="G35" s="9">
+      <c r="G35" s="10">
         <f>G34+F35</f>
         <v/>
       </c>
@@ -1917,34 +2050,34 @@
           <t>À mi-parcours</t>
         </is>
       </c>
-      <c r="J35" s="15" t="n">
+      <c r="J35" s="16" t="n">
         <v>0.4</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="13" t="n">
+      <c r="A36" s="14" t="n">
         <v>46508</v>
       </c>
-      <c r="B36" s="14" t="n">
+      <c r="B36" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="C36" s="9">
+      <c r="C36" s="10">
         <f>IF(2=0+$J$37,$B$19*$J$34,0)+IF(2=3+$J$37,$B$19*$J$35,0)+IF(2=5+$J$37,$B$19*$J$36,0)</f>
         <v/>
       </c>
-      <c r="D36" s="9">
+      <c r="D36" s="10">
         <f>-B36*$B$9</f>
         <v/>
       </c>
-      <c r="E36" s="9">
+      <c r="E36" s="10">
         <f>-($B$21+$B$22+$B$23+$B$24+$B$25+$B$26)/6</f>
         <v/>
       </c>
-      <c r="F36" s="9">
+      <c r="F36" s="10">
         <f>C36+D36+E36</f>
         <v/>
       </c>
-      <c r="G36" s="9">
+      <c r="G36" s="10">
         <f>G35+F36</f>
         <v/>
       </c>
@@ -1953,34 +2086,34 @@
           <t>À la fin</t>
         </is>
       </c>
-      <c r="J36" s="15" t="n">
+      <c r="J36" s="16" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="n">
+      <c r="A37" s="14" t="n">
         <v>46539</v>
       </c>
-      <c r="B37" s="14" t="n">
+      <c r="B37" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="C37" s="9">
+      <c r="C37" s="10">
         <f>IF(3=0+$J$37,$B$19*$J$34,0)+IF(3=3+$J$37,$B$19*$J$35,0)+IF(3=5+$J$37,$B$19*$J$36,0)</f>
         <v/>
       </c>
-      <c r="D37" s="9">
+      <c r="D37" s="10">
         <f>-B37*$B$9</f>
         <v/>
       </c>
-      <c r="E37" s="9">
+      <c r="E37" s="10">
         <f>-($B$21+$B$22+$B$23+$B$24+$B$25+$B$26)/6</f>
         <v/>
       </c>
-      <c r="F37" s="9">
+      <c r="F37" s="10">
         <f>C37+D37+E37</f>
         <v/>
       </c>
-      <c r="G37" s="9">
+      <c r="G37" s="10">
         <f>G36+F37</f>
         <v/>
       </c>
@@ -1989,62 +2122,62 @@
           <t>Délai moyen de paiement (mois)</t>
         </is>
       </c>
-      <c r="J37" s="16" t="n">
+      <c r="J37" s="17" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="n">
+      <c r="A38" s="14" t="n">
         <v>46569</v>
       </c>
-      <c r="B38" s="14" t="n">
+      <c r="B38" s="15" t="n">
         <v>9</v>
       </c>
-      <c r="C38" s="9">
+      <c r="C38" s="10">
         <f>IF(4=0+$J$37,$B$19*$J$34,0)+IF(4=3+$J$37,$B$19*$J$35,0)+IF(4=5+$J$37,$B$19*$J$36,0)</f>
         <v/>
       </c>
-      <c r="D38" s="9">
+      <c r="D38" s="10">
         <f>-B38*$B$9</f>
         <v/>
       </c>
-      <c r="E38" s="9">
+      <c r="E38" s="10">
         <f>-($B$21+$B$22+$B$23+$B$24+$B$25+$B$26)/6</f>
         <v/>
       </c>
-      <c r="F38" s="9">
+      <c r="F38" s="10">
         <f>C38+D38+E38</f>
         <v/>
       </c>
-      <c r="G38" s="9">
+      <c r="G38" s="10">
         <f>G37+F38</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="n">
+      <c r="A39" s="14" t="n">
         <v>46600</v>
       </c>
-      <c r="B39" s="14" t="n">
+      <c r="B39" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="C39" s="9">
+      <c r="C39" s="10">
         <f>IF(5=0+$J$37,$B$19*$J$34,0)+IF(5=3+$J$37,$B$19*$J$35,0)+IF(5=5+$J$37,$B$19*$J$36,0)</f>
         <v/>
       </c>
-      <c r="D39" s="9">
+      <c r="D39" s="10">
         <f>-B39*$B$9</f>
         <v/>
       </c>
-      <c r="E39" s="9">
+      <c r="E39" s="10">
         <f>-($B$21+$B$22+$B$23+$B$24+$B$25+$B$26)/6</f>
         <v/>
       </c>
-      <c r="F39" s="9">
+      <c r="F39" s="10">
         <f>C39+D39+E39</f>
         <v/>
       </c>
-      <c r="G39" s="9">
+      <c r="G39" s="10">
         <f>G38+F39</f>
         <v/>
       </c>
@@ -2055,24 +2188,24 @@
           <t>Mois + 1 après la fin</t>
         </is>
       </c>
-      <c r="B40" s="14" t="n">
+      <c r="B40" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="C40" s="9">
+      <c r="C40" s="10">
         <f>IF(6=0+$J$37,$B$19*$J$34,0)+IF(6=3+$J$37,$B$19*$J$35,0)+IF(6=5+$J$37,$B$19*$J$36,0)</f>
         <v/>
       </c>
-      <c r="D40" s="9" t="n">
+      <c r="D40" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="E40" s="9" t="n">
+      <c r="E40" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F40" s="9">
+      <c r="F40" s="10">
         <f>C40+D40+E40</f>
         <v/>
       </c>
-      <c r="G40" s="9">
+      <c r="G40" s="10">
         <f>G39+F40</f>
         <v/>
       </c>
@@ -2083,24 +2216,24 @@
           <t>Mois + 2 après la fin</t>
         </is>
       </c>
-      <c r="B41" s="14" t="n">
+      <c r="B41" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="C41" s="9">
+      <c r="C41" s="10">
         <f>IF(7=0+$J$37,$B$19*$J$34,0)+IF(7=3+$J$37,$B$19*$J$35,0)+IF(7=5+$J$37,$B$19*$J$36,0)</f>
         <v/>
       </c>
-      <c r="D41" s="9" t="n">
+      <c r="D41" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="E41" s="9" t="n">
+      <c r="E41" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F41" s="9">
+      <c r="F41" s="10">
         <f>C41+D41+E41</f>
         <v/>
       </c>
-      <c r="G41" s="9">
+      <c r="G41" s="10">
         <f>G40+F41</f>
         <v/>
       </c>
@@ -2145,6 +2278,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>TVA : franchise en base (art. 293 B du CGI). Si le chiffre d'affaires annuel dépasse le seuil de franchise, la formation reste sans TVA uniquement avec l'attestation 3511-SD — à voir avec l'expert-comptable.</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -2168,7 +2308,7 @@
           <t>Nombre de stagiaires</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="7" t="n">
         <v>10</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -2183,7 +2323,7 @@
           <t>Prix du parcours par stagiaire</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n"/>
+      <c r="B6" s="8" t="n"/>
       <c r="C6" s="3" t="inlineStr">
         <is>
           <t>[À COMPLÉTER] — prix de vente, net de TVA</t>
@@ -2196,7 +2336,7 @@
           <t>Heures en centre</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="9" t="n">
         <v>595</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -2211,7 +2351,7 @@
           <t>Journées en centre</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="9" t="n">
         <v>85</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -2226,7 +2366,7 @@
           <t>Location de salle par jour</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="8" t="n">
         <v>100</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -2241,7 +2381,7 @@
           <t>Heures assurées par des formateurs externes</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="7" t="n">
         <v>0</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -2256,7 +2396,7 @@
           <t>Coût horaire d'un formateur externe</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n"/>
+      <c r="B11" s="8" t="n"/>
       <c r="C11" s="3" t="inlineStr">
         <is>
           <t>[À COMPLÉTER]</t>
@@ -2269,7 +2409,7 @@
           <t>Ordinateurs portables (achat ou location)</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n"/>
+      <c r="B12" s="8" t="n"/>
       <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Indispensables pour T2 et l'épreuve de mise en situation du MEM</t>
@@ -2282,7 +2422,7 @@
           <t>Coût d'examen par candidat (centre agréé partenaire)</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n"/>
+      <c r="B13" s="8" t="n"/>
       <c r="C13" s="3" t="inlineStr">
         <is>
           <t>[À COMPLÉTER] si pas d'agrément propre</t>
@@ -2295,7 +2435,7 @@
           <t>Jury blanc (défraiement)</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n"/>
+      <c r="B14" s="8" t="n"/>
       <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Professionnels invités</t>
@@ -2308,7 +2448,7 @@
           <t>Communication et recrutement</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n"/>
+      <c r="B15" s="8" t="n"/>
       <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Informations collectives, supports</t>
@@ -2321,7 +2461,7 @@
           <t>Assurances, logiciels, frais administratifs</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n"/>
+      <c r="B16" s="8" t="n"/>
       <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Quote-part de la promotion</t>
@@ -2351,7 +2491,7 @@
           <t>Chiffre d'affaires</t>
         </is>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="10">
         <f>B5*B6</f>
         <v/>
       </c>
@@ -2367,7 +2507,7 @@
           <t>Location de salle</t>
         </is>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="10">
         <f>B8*B9</f>
         <v/>
       </c>
@@ -2383,7 +2523,7 @@
           <t>Formateurs externes</t>
         </is>
       </c>
-      <c r="B21" s="9">
+      <c r="B21" s="10">
         <f>B10*B11</f>
         <v/>
       </c>
@@ -2399,7 +2539,7 @@
           <t>Matériel informatique</t>
         </is>
       </c>
-      <c r="B22" s="9">
+      <c r="B22" s="10">
         <f>B12</f>
         <v/>
       </c>
@@ -2411,7 +2551,7 @@
           <t>Examens</t>
         </is>
       </c>
-      <c r="B23" s="9">
+      <c r="B23" s="10">
         <f>B5*B13</f>
         <v/>
       </c>
@@ -2427,7 +2567,7 @@
           <t>Jury blanc</t>
         </is>
       </c>
-      <c r="B24" s="9">
+      <c r="B24" s="10">
         <f>B14</f>
         <v/>
       </c>
@@ -2439,7 +2579,7 @@
           <t>Communication</t>
         </is>
       </c>
-      <c r="B25" s="9">
+      <c r="B25" s="10">
         <f>B15</f>
         <v/>
       </c>
@@ -2451,31 +2591,31 @@
           <t>Frais généraux</t>
         </is>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="10">
         <f>B16</f>
         <v/>
       </c>
       <c r="C26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>Total des charges</t>
         </is>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="10">
         <f>SUM(B20:B26)</f>
         <v/>
       </c>
       <c r="C27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="inlineStr">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>Résultat de la promotion</t>
         </is>
       </c>
-      <c r="B28" s="9">
+      <c r="B28" s="10">
         <f>B19-B27</f>
         <v/>
       </c>
@@ -2486,12 +2626,12 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="inlineStr">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Seuil de rentabilité (stagiaires)</t>
         </is>
       </c>
-      <c r="B29" s="8">
+      <c r="B29" s="9">
         <f>IF(B6&gt;0,ROUNDUP((B27-B5*B13)/(B6-B13),0),"")</f>
         <v/>
       </c>
@@ -2507,7 +2647,7 @@
           <t>Coût de la salle par heure-stagiaire</t>
         </is>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="12">
         <f>IF(B5&gt;0,B20/(B7*B5),"")</f>
         <v/>
       </c>
@@ -2553,36 +2693,36 @@
           <t>Solde cumulé</t>
         </is>
       </c>
-      <c r="I33" s="12" t="inlineStr">
+      <c r="I33" s="13" t="inlineStr">
         <is>
           <t>Échéancier d'encaissement</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="n">
+      <c r="A34" s="14" t="n">
         <v>46631</v>
       </c>
-      <c r="B34" s="14" t="n">
+      <c r="B34" s="15" t="n">
         <v>19</v>
       </c>
-      <c r="C34" s="9">
+      <c r="C34" s="10">
         <f>IF(0=0+$J$37,$B$19*$J$34,0)+IF(0=3+$J$37,$B$19*$J$35,0)+IF(0=5+$J$37,$B$19*$J$36,0)</f>
         <v/>
       </c>
-      <c r="D34" s="9">
+      <c r="D34" s="10">
         <f>-B34*$B$9</f>
         <v/>
       </c>
-      <c r="E34" s="9">
+      <c r="E34" s="10">
         <f>-($B$21+$B$22+$B$23+$B$24+$B$25+$B$26)/6</f>
         <v/>
       </c>
-      <c r="F34" s="9">
+      <c r="F34" s="10">
         <f>C34+D34+E34</f>
         <v/>
       </c>
-      <c r="G34" s="9">
+      <c r="G34" s="10">
         <f>F34</f>
         <v/>
       </c>
@@ -2591,34 +2731,34 @@
           <t>À l'entrée</t>
         </is>
       </c>
-      <c r="J34" s="15" t="n">
+      <c r="J34" s="16" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="n">
+      <c r="A35" s="14" t="n">
         <v>46661</v>
       </c>
-      <c r="B35" s="14" t="n">
+      <c r="B35" s="15" t="n">
         <v>21</v>
       </c>
-      <c r="C35" s="9">
+      <c r="C35" s="10">
         <f>IF(1=0+$J$37,$B$19*$J$34,0)+IF(1=3+$J$37,$B$19*$J$35,0)+IF(1=5+$J$37,$B$19*$J$36,0)</f>
         <v/>
       </c>
-      <c r="D35" s="9">
+      <c r="D35" s="10">
         <f>-B35*$B$9</f>
         <v/>
       </c>
-      <c r="E35" s="9">
+      <c r="E35" s="10">
         <f>-($B$21+$B$22+$B$23+$B$24+$B$25+$B$26)/6</f>
         <v/>
       </c>
-      <c r="F35" s="9">
+      <c r="F35" s="10">
         <f>C35+D35+E35</f>
         <v/>
       </c>
-      <c r="G35" s="9">
+      <c r="G35" s="10">
         <f>G34+F35</f>
         <v/>
       </c>
@@ -2627,34 +2767,34 @@
           <t>À mi-parcours</t>
         </is>
       </c>
-      <c r="J35" s="15" t="n">
+      <c r="J35" s="16" t="n">
         <v>0.4</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="13" t="n">
+      <c r="A36" s="14" t="n">
         <v>46692</v>
       </c>
-      <c r="B36" s="14" t="n">
+      <c r="B36" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="C36" s="9">
+      <c r="C36" s="10">
         <f>IF(2=0+$J$37,$B$19*$J$34,0)+IF(2=3+$J$37,$B$19*$J$35,0)+IF(2=5+$J$37,$B$19*$J$36,0)</f>
         <v/>
       </c>
-      <c r="D36" s="9">
+      <c r="D36" s="10">
         <f>-B36*$B$9</f>
         <v/>
       </c>
-      <c r="E36" s="9">
+      <c r="E36" s="10">
         <f>-($B$21+$B$22+$B$23+$B$24+$B$25+$B$26)/6</f>
         <v/>
       </c>
-      <c r="F36" s="9">
+      <c r="F36" s="10">
         <f>C36+D36+E36</f>
         <v/>
       </c>
-      <c r="G36" s="9">
+      <c r="G36" s="10">
         <f>G35+F36</f>
         <v/>
       </c>
@@ -2663,34 +2803,34 @@
           <t>À la fin</t>
         </is>
       </c>
-      <c r="J36" s="15" t="n">
+      <c r="J36" s="16" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="n">
+      <c r="A37" s="14" t="n">
         <v>46722</v>
       </c>
-      <c r="B37" s="14" t="n">
+      <c r="B37" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="C37" s="9">
+      <c r="C37" s="10">
         <f>IF(3=0+$J$37,$B$19*$J$34,0)+IF(3=3+$J$37,$B$19*$J$35,0)+IF(3=5+$J$37,$B$19*$J$36,0)</f>
         <v/>
       </c>
-      <c r="D37" s="9">
+      <c r="D37" s="10">
         <f>-B37*$B$9</f>
         <v/>
       </c>
-      <c r="E37" s="9">
+      <c r="E37" s="10">
         <f>-($B$21+$B$22+$B$23+$B$24+$B$25+$B$26)/6</f>
         <v/>
       </c>
-      <c r="F37" s="9">
+      <c r="F37" s="10">
         <f>C37+D37+E37</f>
         <v/>
       </c>
-      <c r="G37" s="9">
+      <c r="G37" s="10">
         <f>G36+F37</f>
         <v/>
       </c>
@@ -2699,62 +2839,62 @@
           <t>Délai moyen de paiement (mois)</t>
         </is>
       </c>
-      <c r="J37" s="16" t="n">
+      <c r="J37" s="17" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="n">
+      <c r="A38" s="14" t="n">
         <v>46753</v>
       </c>
-      <c r="B38" s="14" t="n">
+      <c r="B38" s="15" t="n">
         <v>21</v>
       </c>
-      <c r="C38" s="9">
+      <c r="C38" s="10">
         <f>IF(4=0+$J$37,$B$19*$J$34,0)+IF(4=3+$J$37,$B$19*$J$35,0)+IF(4=5+$J$37,$B$19*$J$36,0)</f>
         <v/>
       </c>
-      <c r="D38" s="9">
+      <c r="D38" s="10">
         <f>-B38*$B$9</f>
         <v/>
       </c>
-      <c r="E38" s="9">
+      <c r="E38" s="10">
         <f>-($B$21+$B$22+$B$23+$B$24+$B$25+$B$26)/6</f>
         <v/>
       </c>
-      <c r="F38" s="9">
+      <c r="F38" s="10">
         <f>C38+D38+E38</f>
         <v/>
       </c>
-      <c r="G38" s="9">
+      <c r="G38" s="10">
         <f>G37+F38</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="n">
+      <c r="A39" s="14" t="n">
         <v>46784</v>
       </c>
-      <c r="B39" s="14" t="n">
+      <c r="B39" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="C39" s="9">
+      <c r="C39" s="10">
         <f>IF(5=0+$J$37,$B$19*$J$34,0)+IF(5=3+$J$37,$B$19*$J$35,0)+IF(5=5+$J$37,$B$19*$J$36,0)</f>
         <v/>
       </c>
-      <c r="D39" s="9">
+      <c r="D39" s="10">
         <f>-B39*$B$9</f>
         <v/>
       </c>
-      <c r="E39" s="9">
+      <c r="E39" s="10">
         <f>-($B$21+$B$22+$B$23+$B$24+$B$25+$B$26)/6</f>
         <v/>
       </c>
-      <c r="F39" s="9">
+      <c r="F39" s="10">
         <f>C39+D39+E39</f>
         <v/>
       </c>
-      <c r="G39" s="9">
+      <c r="G39" s="10">
         <f>G38+F39</f>
         <v/>
       </c>
@@ -2765,24 +2905,24 @@
           <t>Mois + 1 après la fin</t>
         </is>
       </c>
-      <c r="B40" s="14" t="n">
+      <c r="B40" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="C40" s="9">
+      <c r="C40" s="10">
         <f>IF(6=0+$J$37,$B$19*$J$34,0)+IF(6=3+$J$37,$B$19*$J$35,0)+IF(6=5+$J$37,$B$19*$J$36,0)</f>
         <v/>
       </c>
-      <c r="D40" s="9" t="n">
+      <c r="D40" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="E40" s="9" t="n">
+      <c r="E40" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F40" s="9">
+      <c r="F40" s="10">
         <f>C40+D40+E40</f>
         <v/>
       </c>
-      <c r="G40" s="9">
+      <c r="G40" s="10">
         <f>G39+F40</f>
         <v/>
       </c>
@@ -2793,24 +2933,24 @@
           <t>Mois + 2 après la fin</t>
         </is>
       </c>
-      <c r="B41" s="14" t="n">
+      <c r="B41" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="C41" s="9">
+      <c r="C41" s="10">
         <f>IF(7=0+$J$37,$B$19*$J$34,0)+IF(7=3+$J$37,$B$19*$J$35,0)+IF(7=5+$J$37,$B$19*$J$36,0)</f>
         <v/>
       </c>
-      <c r="D41" s="9" t="n">
+      <c r="D41" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="E41" s="9" t="n">
+      <c r="E41" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F41" s="9">
+      <c r="F41" s="10">
         <f>C41+D41+E41</f>
         <v/>
       </c>
-      <c r="G41" s="9">
+      <c r="G41" s="10">
         <f>G40+F41</f>
         <v/>
       </c>
@@ -2897,7 +3037,7 @@
       <c r="E2" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F2" s="17" t="n"/>
+      <c r="F2" s="18" t="n"/>
       <c r="G2" s="3">
         <f>IF(F2="","",F2-E2)</f>
         <v/>
@@ -2925,7 +3065,7 @@
       <c r="E3" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F3" s="17" t="n"/>
+      <c r="F3" s="18" t="n"/>
       <c r="G3" s="3">
         <f>IF(F3="","",F3-E3)</f>
         <v/>
@@ -2953,7 +3093,7 @@
       <c r="E4" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F4" s="17" t="n"/>
+      <c r="F4" s="18" t="n"/>
       <c r="G4" s="3">
         <f>IF(F4="","",F4-E4)</f>
         <v/>
@@ -2981,7 +3121,7 @@
       <c r="E5" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F5" s="17" t="n"/>
+      <c r="F5" s="18" t="n"/>
       <c r="G5" s="3">
         <f>IF(F5="","",F5-E5)</f>
         <v/>
@@ -3009,7 +3149,7 @@
       <c r="E6" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F6" s="17" t="n"/>
+      <c r="F6" s="18" t="n"/>
       <c r="G6" s="3">
         <f>IF(F6="","",F6-E6)</f>
         <v/>
@@ -3037,7 +3177,7 @@
       <c r="E7" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F7" s="17" t="n"/>
+      <c r="F7" s="18" t="n"/>
       <c r="G7" s="3">
         <f>IF(F7="","",F7-E7)</f>
         <v/>
@@ -3065,7 +3205,7 @@
       <c r="E8" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F8" s="17" t="n"/>
+      <c r="F8" s="18" t="n"/>
       <c r="G8" s="3">
         <f>IF(F8="","",F8-E8)</f>
         <v/>
@@ -3093,7 +3233,7 @@
       <c r="E9" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F9" s="17" t="n"/>
+      <c r="F9" s="18" t="n"/>
       <c r="G9" s="3">
         <f>IF(F9="","",F9-E9)</f>
         <v/>
@@ -3121,7 +3261,7 @@
       <c r="E10" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F10" s="17" t="n"/>
+      <c r="F10" s="18" t="n"/>
       <c r="G10" s="3">
         <f>IF(F10="","",F10-E10)</f>
         <v/>
@@ -3149,7 +3289,7 @@
       <c r="E11" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F11" s="17" t="n"/>
+      <c r="F11" s="18" t="n"/>
       <c r="G11" s="3">
         <f>IF(F11="","",F11-E11)</f>
         <v/>
@@ -3177,7 +3317,7 @@
       <c r="E12" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F12" s="17" t="n"/>
+      <c r="F12" s="18" t="n"/>
       <c r="G12" s="3">
         <f>IF(F12="","",F12-E12)</f>
         <v/>
@@ -3205,7 +3345,7 @@
       <c r="E13" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F13" s="17" t="n"/>
+      <c r="F13" s="18" t="n"/>
       <c r="G13" s="3">
         <f>IF(F13="","",F13-E13)</f>
         <v/>
@@ -3233,7 +3373,7 @@
       <c r="E14" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F14" s="17" t="n"/>
+      <c r="F14" s="18" t="n"/>
       <c r="G14" s="3">
         <f>IF(F14="","",F14-E14)</f>
         <v/>
@@ -3261,7 +3401,7 @@
       <c r="E15" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F15" s="17" t="n"/>
+      <c r="F15" s="18" t="n"/>
       <c r="G15" s="3">
         <f>IF(F15="","",F15-E15)</f>
         <v/>
@@ -3289,7 +3429,7 @@
       <c r="E16" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F16" s="17" t="n"/>
+      <c r="F16" s="18" t="n"/>
       <c r="G16" s="3">
         <f>IF(F16="","",F16-E16)</f>
         <v/>
@@ -3317,7 +3457,7 @@
       <c r="E17" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F17" s="17" t="n"/>
+      <c r="F17" s="18" t="n"/>
       <c r="G17" s="3">
         <f>IF(F17="","",F17-E17)</f>
         <v/>
@@ -3345,7 +3485,7 @@
       <c r="E18" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F18" s="17" t="n"/>
+      <c r="F18" s="18" t="n"/>
       <c r="G18" s="3">
         <f>IF(F18="","",F18-E18)</f>
         <v/>
@@ -3373,7 +3513,7 @@
       <c r="E19" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F19" s="17" t="n"/>
+      <c r="F19" s="18" t="n"/>
       <c r="G19" s="3">
         <f>IF(F19="","",F19-E19)</f>
         <v/>
@@ -3401,7 +3541,7 @@
       <c r="E20" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F20" s="17" t="n"/>
+      <c r="F20" s="18" t="n"/>
       <c r="G20" s="3">
         <f>IF(F20="","",F20-E20)</f>
         <v/>
@@ -3429,7 +3569,7 @@
       <c r="E21" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F21" s="17" t="n"/>
+      <c r="F21" s="18" t="n"/>
       <c r="G21" s="3">
         <f>IF(F21="","",F21-E21)</f>
         <v/>
@@ -3457,7 +3597,7 @@
       <c r="E22" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F22" s="17" t="n"/>
+      <c r="F22" s="18" t="n"/>
       <c r="G22" s="3">
         <f>IF(F22="","",F22-E22)</f>
         <v/>
@@ -3485,7 +3625,7 @@
       <c r="E23" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F23" s="17" t="n"/>
+      <c r="F23" s="18" t="n"/>
       <c r="G23" s="3">
         <f>IF(F23="","",F23-E23)</f>
         <v/>
@@ -3513,7 +3653,7 @@
       <c r="E24" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F24" s="17" t="n"/>
+      <c r="F24" s="18" t="n"/>
       <c r="G24" s="3">
         <f>IF(F24="","",F24-E24)</f>
         <v/>
@@ -3541,7 +3681,7 @@
       <c r="E25" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F25" s="17" t="n"/>
+      <c r="F25" s="18" t="n"/>
       <c r="G25" s="3">
         <f>IF(F25="","",F25-E25)</f>
         <v/>
@@ -3569,7 +3709,7 @@
       <c r="E26" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F26" s="17" t="n"/>
+      <c r="F26" s="18" t="n"/>
       <c r="G26" s="3">
         <f>IF(F26="","",F26-E26)</f>
         <v/>
@@ -3597,7 +3737,7 @@
       <c r="E27" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F27" s="17" t="n"/>
+      <c r="F27" s="18" t="n"/>
       <c r="G27" s="3">
         <f>IF(F27="","",F27-E27)</f>
         <v/>
@@ -3625,7 +3765,7 @@
       <c r="E28" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F28" s="17" t="n"/>
+      <c r="F28" s="18" t="n"/>
       <c r="G28" s="3">
         <f>IF(F28="","",F28-E28)</f>
         <v/>
@@ -3653,7 +3793,7 @@
       <c r="E29" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F29" s="17" t="n"/>
+      <c r="F29" s="18" t="n"/>
       <c r="G29" s="3">
         <f>IF(F29="","",F29-E29)</f>
         <v/>
@@ -3681,7 +3821,7 @@
       <c r="E30" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F30" s="17" t="n"/>
+      <c r="F30" s="18" t="n"/>
       <c r="G30" s="3">
         <f>IF(F30="","",F30-E30)</f>
         <v/>
@@ -3709,7 +3849,7 @@
       <c r="E31" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F31" s="17" t="n"/>
+      <c r="F31" s="18" t="n"/>
       <c r="G31" s="3">
         <f>IF(F31="","",F31-E31)</f>
         <v/>
@@ -3737,7 +3877,7 @@
       <c r="E32" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F32" s="17" t="n"/>
+      <c r="F32" s="18" t="n"/>
       <c r="G32" s="3">
         <f>IF(F32="","",F32-E32)</f>
         <v/>
@@ -3765,7 +3905,7 @@
       <c r="E33" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F33" s="17" t="n"/>
+      <c r="F33" s="18" t="n"/>
       <c r="G33" s="3">
         <f>IF(F33="","",F33-E33)</f>
         <v/>
@@ -3793,7 +3933,7 @@
       <c r="E34" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F34" s="17" t="n"/>
+      <c r="F34" s="18" t="n"/>
       <c r="G34" s="3">
         <f>IF(F34="","",F34-E34)</f>
         <v/>
@@ -3821,7 +3961,7 @@
       <c r="E35" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F35" s="17" t="n"/>
+      <c r="F35" s="18" t="n"/>
       <c r="G35" s="3">
         <f>IF(F35="","",F35-E35)</f>
         <v/>
@@ -3849,7 +3989,7 @@
       <c r="E36" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F36" s="17" t="n"/>
+      <c r="F36" s="18" t="n"/>
       <c r="G36" s="3">
         <f>IF(F36="","",F36-E36)</f>
         <v/>
@@ -3877,7 +4017,7 @@
       <c r="E37" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F37" s="17" t="n"/>
+      <c r="F37" s="18" t="n"/>
       <c r="G37" s="3">
         <f>IF(F37="","",F37-E37)</f>
         <v/>
@@ -3905,7 +4045,7 @@
       <c r="E38" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F38" s="17" t="n"/>
+      <c r="F38" s="18" t="n"/>
       <c r="G38" s="3">
         <f>IF(F38="","",F38-E38)</f>
         <v/>
@@ -3933,7 +4073,7 @@
       <c r="E39" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F39" s="17" t="n"/>
+      <c r="F39" s="18" t="n"/>
       <c r="G39" s="3">
         <f>IF(F39="","",F39-E39)</f>
         <v/>
@@ -3961,7 +4101,7 @@
       <c r="E40" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F40" s="17" t="n"/>
+      <c r="F40" s="18" t="n"/>
       <c r="G40" s="3">
         <f>IF(F40="","",F40-E40)</f>
         <v/>
@@ -3989,7 +4129,7 @@
       <c r="E41" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F41" s="17" t="n"/>
+      <c r="F41" s="18" t="n"/>
       <c r="G41" s="3">
         <f>IF(F41="","",F41-E41)</f>
         <v/>
@@ -4017,7 +4157,7 @@
       <c r="E42" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F42" s="17" t="n"/>
+      <c r="F42" s="18" t="n"/>
       <c r="G42" s="3">
         <f>IF(F42="","",F42-E42)</f>
         <v/>
@@ -4045,7 +4185,7 @@
       <c r="E43" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F43" s="17" t="n"/>
+      <c r="F43" s="18" t="n"/>
       <c r="G43" s="3">
         <f>IF(F43="","",F43-E43)</f>
         <v/>
@@ -4073,7 +4213,7 @@
       <c r="E44" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F44" s="17" t="n"/>
+      <c r="F44" s="18" t="n"/>
       <c r="G44" s="3">
         <f>IF(F44="","",F44-E44)</f>
         <v/>
@@ -4101,7 +4241,7 @@
       <c r="E45" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F45" s="17" t="n"/>
+      <c r="F45" s="18" t="n"/>
       <c r="G45" s="3">
         <f>IF(F45="","",F45-E45)</f>
         <v/>
@@ -4129,7 +4269,7 @@
       <c r="E46" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F46" s="17" t="n"/>
+      <c r="F46" s="18" t="n"/>
       <c r="G46" s="3">
         <f>IF(F46="","",F46-E46)</f>
         <v/>
@@ -4157,7 +4297,7 @@
       <c r="E47" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F47" s="17" t="n"/>
+      <c r="F47" s="18" t="n"/>
       <c r="G47" s="3">
         <f>IF(F47="","",F47-E47)</f>
         <v/>
@@ -4185,7 +4325,7 @@
       <c r="E48" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F48" s="17" t="n"/>
+      <c r="F48" s="18" t="n"/>
       <c r="G48" s="3">
         <f>IF(F48="","",F48-E48)</f>
         <v/>
@@ -4213,7 +4353,7 @@
       <c r="E49" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F49" s="17" t="n"/>
+      <c r="F49" s="18" t="n"/>
       <c r="G49" s="3">
         <f>IF(F49="","",F49-E49)</f>
         <v/>
@@ -4241,7 +4381,7 @@
       <c r="E50" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F50" s="17" t="n"/>
+      <c r="F50" s="18" t="n"/>
       <c r="G50" s="3">
         <f>IF(F50="","",F50-E50)</f>
         <v/>
@@ -4269,7 +4409,7 @@
       <c r="E51" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F51" s="17" t="n"/>
+      <c r="F51" s="18" t="n"/>
       <c r="G51" s="3">
         <f>IF(F51="","",F51-E51)</f>
         <v/>
@@ -4297,7 +4437,7 @@
       <c r="E52" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F52" s="17" t="n"/>
+      <c r="F52" s="18" t="n"/>
       <c r="G52" s="3">
         <f>IF(F52="","",F52-E52)</f>
         <v/>
@@ -4325,7 +4465,7 @@
       <c r="E53" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F53" s="17" t="n"/>
+      <c r="F53" s="18" t="n"/>
       <c r="G53" s="3">
         <f>IF(F53="","",F53-E53)</f>
         <v/>
@@ -4353,7 +4493,7 @@
       <c r="E54" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F54" s="17" t="n"/>
+      <c r="F54" s="18" t="n"/>
       <c r="G54" s="3">
         <f>IF(F54="","",F54-E54)</f>
         <v/>
@@ -4381,7 +4521,7 @@
       <c r="E55" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F55" s="17" t="n"/>
+      <c r="F55" s="18" t="n"/>
       <c r="G55" s="3">
         <f>IF(F55="","",F55-E55)</f>
         <v/>
@@ -4409,7 +4549,7 @@
       <c r="E56" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F56" s="17" t="n"/>
+      <c r="F56" s="18" t="n"/>
       <c r="G56" s="3">
         <f>IF(F56="","",F56-E56)</f>
         <v/>
@@ -4437,7 +4577,7 @@
       <c r="E57" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F57" s="17" t="n"/>
+      <c r="F57" s="18" t="n"/>
       <c r="G57" s="3">
         <f>IF(F57="","",F57-E57)</f>
         <v/>
@@ -4465,7 +4605,7 @@
       <c r="E58" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F58" s="17" t="n"/>
+      <c r="F58" s="18" t="n"/>
       <c r="G58" s="3">
         <f>IF(F58="","",F58-E58)</f>
         <v/>
@@ -4493,7 +4633,7 @@
       <c r="E59" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F59" s="17" t="n"/>
+      <c r="F59" s="18" t="n"/>
       <c r="G59" s="3">
         <f>IF(F59="","",F59-E59)</f>
         <v/>
@@ -4521,7 +4661,7 @@
       <c r="E60" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F60" s="17" t="n"/>
+      <c r="F60" s="18" t="n"/>
       <c r="G60" s="3">
         <f>IF(F60="","",F60-E60)</f>
         <v/>
@@ -4549,7 +4689,7 @@
       <c r="E61" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F61" s="17" t="n"/>
+      <c r="F61" s="18" t="n"/>
       <c r="G61" s="3">
         <f>IF(F61="","",F61-E61)</f>
         <v/>
@@ -4577,7 +4717,7 @@
       <c r="E62" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F62" s="17" t="n"/>
+      <c r="F62" s="18" t="n"/>
       <c r="G62" s="3">
         <f>IF(F62="","",F62-E62)</f>
         <v/>
@@ -4605,7 +4745,7 @@
       <c r="E63" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F63" s="17" t="n"/>
+      <c r="F63" s="18" t="n"/>
       <c r="G63" s="3">
         <f>IF(F63="","",F63-E63)</f>
         <v/>
@@ -4633,7 +4773,7 @@
       <c r="E64" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F64" s="17" t="n"/>
+      <c r="F64" s="18" t="n"/>
       <c r="G64" s="3">
         <f>IF(F64="","",F64-E64)</f>
         <v/>
@@ -4661,7 +4801,7 @@
       <c r="E65" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F65" s="17" t="n"/>
+      <c r="F65" s="18" t="n"/>
       <c r="G65" s="3">
         <f>IF(F65="","",F65-E65)</f>
         <v/>
@@ -4689,7 +4829,7 @@
       <c r="E66" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F66" s="17" t="n"/>
+      <c r="F66" s="18" t="n"/>
       <c r="G66" s="3">
         <f>IF(F66="","",F66-E66)</f>
         <v/>
@@ -4717,7 +4857,7 @@
       <c r="E67" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F67" s="17" t="n"/>
+      <c r="F67" s="18" t="n"/>
       <c r="G67" s="3">
         <f>IF(F67="","",F67-E67)</f>
         <v/>
@@ -4745,7 +4885,7 @@
       <c r="E68" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F68" s="17" t="n"/>
+      <c r="F68" s="18" t="n"/>
       <c r="G68" s="3">
         <f>IF(F68="","",F68-E68)</f>
         <v/>
@@ -4773,7 +4913,7 @@
       <c r="E69" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F69" s="17" t="n"/>
+      <c r="F69" s="18" t="n"/>
       <c r="G69" s="3">
         <f>IF(F69="","",F69-E69)</f>
         <v/>
@@ -4801,7 +4941,7 @@
       <c r="E70" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F70" s="17" t="n"/>
+      <c r="F70" s="18" t="n"/>
       <c r="G70" s="3">
         <f>IF(F70="","",F70-E70)</f>
         <v/>
@@ -4829,7 +4969,7 @@
       <c r="E71" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F71" s="17" t="n"/>
+      <c r="F71" s="18" t="n"/>
       <c r="G71" s="3">
         <f>IF(F71="","",F71-E71)</f>
         <v/>
@@ -4857,7 +4997,7 @@
       <c r="E72" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F72" s="17" t="n"/>
+      <c r="F72" s="18" t="n"/>
       <c r="G72" s="3">
         <f>IF(F72="","",F72-E72)</f>
         <v/>
@@ -4885,7 +5025,7 @@
       <c r="E73" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F73" s="17" t="n"/>
+      <c r="F73" s="18" t="n"/>
       <c r="G73" s="3">
         <f>IF(F73="","",F73-E73)</f>
         <v/>
@@ -4913,7 +5053,7 @@
       <c r="E74" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F74" s="17" t="n"/>
+      <c r="F74" s="18" t="n"/>
       <c r="G74" s="3">
         <f>IF(F74="","",F74-E74)</f>
         <v/>
@@ -4941,7 +5081,7 @@
       <c r="E75" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F75" s="17" t="n"/>
+      <c r="F75" s="18" t="n"/>
       <c r="G75" s="3">
         <f>IF(F75="","",F75-E75)</f>
         <v/>
@@ -4969,7 +5109,7 @@
       <c r="E76" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F76" s="17" t="n"/>
+      <c r="F76" s="18" t="n"/>
       <c r="G76" s="3">
         <f>IF(F76="","",F76-E76)</f>
         <v/>
@@ -4997,7 +5137,7 @@
       <c r="E77" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F77" s="17" t="n"/>
+      <c r="F77" s="18" t="n"/>
       <c r="G77" s="3">
         <f>IF(F77="","",F77-E77)</f>
         <v/>
@@ -5025,7 +5165,7 @@
       <c r="E78" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F78" s="17" t="n"/>
+      <c r="F78" s="18" t="n"/>
       <c r="G78" s="3">
         <f>IF(F78="","",F78-E78)</f>
         <v/>
@@ -5053,7 +5193,7 @@
       <c r="E79" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F79" s="17" t="n"/>
+      <c r="F79" s="18" t="n"/>
       <c r="G79" s="3">
         <f>IF(F79="","",F79-E79)</f>
         <v/>
@@ -5081,7 +5221,7 @@
       <c r="E80" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F80" s="17" t="n"/>
+      <c r="F80" s="18" t="n"/>
       <c r="G80" s="3">
         <f>IF(F80="","",F80-E80)</f>
         <v/>
@@ -5109,7 +5249,7 @@
       <c r="E81" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F81" s="17" t="n"/>
+      <c r="F81" s="18" t="n"/>
       <c r="G81" s="3">
         <f>IF(F81="","",F81-E81)</f>
         <v/>
@@ -5137,7 +5277,7 @@
       <c r="E82" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F82" s="17" t="n"/>
+      <c r="F82" s="18" t="n"/>
       <c r="G82" s="3">
         <f>IF(F82="","",F82-E82)</f>
         <v/>
@@ -5165,7 +5305,7 @@
       <c r="E83" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F83" s="17" t="n"/>
+      <c r="F83" s="18" t="n"/>
       <c r="G83" s="3">
         <f>IF(F83="","",F83-E83)</f>
         <v/>
@@ -5193,7 +5333,7 @@
       <c r="E84" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F84" s="17" t="n"/>
+      <c r="F84" s="18" t="n"/>
       <c r="G84" s="3">
         <f>IF(F84="","",F84-E84)</f>
         <v/>
@@ -5221,7 +5361,7 @@
       <c r="E85" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F85" s="17" t="n"/>
+      <c r="F85" s="18" t="n"/>
       <c r="G85" s="3">
         <f>IF(F85="","",F85-E85)</f>
         <v/>
@@ -5249,7 +5389,7 @@
       <c r="E86" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F86" s="17" t="n"/>
+      <c r="F86" s="18" t="n"/>
       <c r="G86" s="3">
         <f>IF(F86="","",F86-E86)</f>
         <v/>
@@ -5277,7 +5417,7 @@
       <c r="E87" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F87" s="17" t="n"/>
+      <c r="F87" s="18" t="n"/>
       <c r="G87" s="3">
         <f>IF(F87="","",F87-E87)</f>
         <v/>
@@ -5305,7 +5445,7 @@
       <c r="E88" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F88" s="17" t="n"/>
+      <c r="F88" s="18" t="n"/>
       <c r="G88" s="3">
         <f>IF(F88="","",F88-E88)</f>
         <v/>
@@ -5333,7 +5473,7 @@
       <c r="E89" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F89" s="17" t="n"/>
+      <c r="F89" s="18" t="n"/>
       <c r="G89" s="3">
         <f>IF(F89="","",F89-E89)</f>
         <v/>
@@ -5361,7 +5501,7 @@
       <c r="E90" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F90" s="17" t="n"/>
+      <c r="F90" s="18" t="n"/>
       <c r="G90" s="3">
         <f>IF(F90="","",F90-E90)</f>
         <v/>
@@ -5389,7 +5529,7 @@
       <c r="E91" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F91" s="17" t="n"/>
+      <c r="F91" s="18" t="n"/>
       <c r="G91" s="3">
         <f>IF(F91="","",F91-E91)</f>
         <v/>
@@ -5417,7 +5557,7 @@
       <c r="E92" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F92" s="17" t="n"/>
+      <c r="F92" s="18" t="n"/>
       <c r="G92" s="3">
         <f>IF(F92="","",F92-E92)</f>
         <v/>
@@ -5445,7 +5585,7 @@
       <c r="E93" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F93" s="17" t="n"/>
+      <c r="F93" s="18" t="n"/>
       <c r="G93" s="3">
         <f>IF(F93="","",F93-E93)</f>
         <v/>
@@ -5473,7 +5613,7 @@
       <c r="E94" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F94" s="17" t="n"/>
+      <c r="F94" s="18" t="n"/>
       <c r="G94" s="3">
         <f>IF(F94="","",F94-E94)</f>
         <v/>
@@ -5501,7 +5641,7 @@
       <c r="E95" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F95" s="17" t="n"/>
+      <c r="F95" s="18" t="n"/>
       <c r="G95" s="3">
         <f>IF(F95="","",F95-E95)</f>
         <v/>
@@ -5529,7 +5669,7 @@
       <c r="E96" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F96" s="17" t="n"/>
+      <c r="F96" s="18" t="n"/>
       <c r="G96" s="3">
         <f>IF(F96="","",F96-E96)</f>
         <v/>
@@ -5557,7 +5697,7 @@
       <c r="E97" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F97" s="17" t="n"/>
+      <c r="F97" s="18" t="n"/>
       <c r="G97" s="3">
         <f>IF(F97="","",F97-E97)</f>
         <v/>
@@ -5585,7 +5725,7 @@
       <c r="E98" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F98" s="17" t="n"/>
+      <c r="F98" s="18" t="n"/>
       <c r="G98" s="3">
         <f>IF(F98="","",F98-E98)</f>
         <v/>
@@ -5613,7 +5753,7 @@
       <c r="E99" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F99" s="17" t="n"/>
+      <c r="F99" s="18" t="n"/>
       <c r="G99" s="3">
         <f>IF(F99="","",F99-E99)</f>
         <v/>
@@ -5641,7 +5781,7 @@
       <c r="E100" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F100" s="17" t="n"/>
+      <c r="F100" s="18" t="n"/>
       <c r="G100" s="3">
         <f>IF(F100="","",F100-E100)</f>
         <v/>
@@ -5669,7 +5809,7 @@
       <c r="E101" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F101" s="17" t="n"/>
+      <c r="F101" s="18" t="n"/>
       <c r="G101" s="3">
         <f>IF(F101="","",F101-E101)</f>
         <v/>
@@ -5697,7 +5837,7 @@
       <c r="E102" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F102" s="17" t="n"/>
+      <c r="F102" s="18" t="n"/>
       <c r="G102" s="3">
         <f>IF(F102="","",F102-E102)</f>
         <v/>
@@ -5725,7 +5865,7 @@
       <c r="E103" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F103" s="17" t="n"/>
+      <c r="F103" s="18" t="n"/>
       <c r="G103" s="3">
         <f>IF(F103="","",F103-E103)</f>
         <v/>
@@ -5753,7 +5893,7 @@
       <c r="E104" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F104" s="17" t="n"/>
+      <c r="F104" s="18" t="n"/>
       <c r="G104" s="3">
         <f>IF(F104="","",F104-E104)</f>
         <v/>
@@ -5781,7 +5921,7 @@
       <c r="E105" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F105" s="17" t="n"/>
+      <c r="F105" s="18" t="n"/>
       <c r="G105" s="3">
         <f>IF(F105="","",F105-E105)</f>
         <v/>
@@ -5809,7 +5949,7 @@
       <c r="E106" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F106" s="17" t="n"/>
+      <c r="F106" s="18" t="n"/>
       <c r="G106" s="3">
         <f>IF(F106="","",F106-E106)</f>
         <v/>
@@ -5837,7 +5977,7 @@
       <c r="E107" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F107" s="17" t="n"/>
+      <c r="F107" s="18" t="n"/>
       <c r="G107" s="3">
         <f>IF(F107="","",F107-E107)</f>
         <v/>
@@ -5865,7 +6005,7 @@
       <c r="E108" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F108" s="17" t="n"/>
+      <c r="F108" s="18" t="n"/>
       <c r="G108" s="3">
         <f>IF(F108="","",F108-E108)</f>
         <v/>
@@ -5893,7 +6033,7 @@
       <c r="E109" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F109" s="17" t="n"/>
+      <c r="F109" s="18" t="n"/>
       <c r="G109" s="3">
         <f>IF(F109="","",F109-E109)</f>
         <v/>
@@ -5921,7 +6061,7 @@
       <c r="E110" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F110" s="17" t="n"/>
+      <c r="F110" s="18" t="n"/>
       <c r="G110" s="3">
         <f>IF(F110="","",F110-E110)</f>
         <v/>
@@ -5949,7 +6089,7 @@
       <c r="E111" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F111" s="17" t="n"/>
+      <c r="F111" s="18" t="n"/>
       <c r="G111" s="3">
         <f>IF(F111="","",F111-E111)</f>
         <v/>
@@ -5977,7 +6117,7 @@
       <c r="E112" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F112" s="17" t="n"/>
+      <c r="F112" s="18" t="n"/>
       <c r="G112" s="3">
         <f>IF(F112="","",F112-E112)</f>
         <v/>
@@ -6005,7 +6145,7 @@
       <c r="E113" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F113" s="17" t="n"/>
+      <c r="F113" s="18" t="n"/>
       <c r="G113" s="3">
         <f>IF(F113="","",F113-E113)</f>
         <v/>
@@ -6033,7 +6173,7 @@
       <c r="E114" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F114" s="17" t="n"/>
+      <c r="F114" s="18" t="n"/>
       <c r="G114" s="3">
         <f>IF(F114="","",F114-E114)</f>
         <v/>
@@ -6061,7 +6201,7 @@
       <c r="E115" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F115" s="17" t="n"/>
+      <c r="F115" s="18" t="n"/>
       <c r="G115" s="3">
         <f>IF(F115="","",F115-E115)</f>
         <v/>
@@ -6089,7 +6229,7 @@
       <c r="E116" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F116" s="17" t="n"/>
+      <c r="F116" s="18" t="n"/>
       <c r="G116" s="3">
         <f>IF(F116="","",F116-E116)</f>
         <v/>
@@ -6117,7 +6257,7 @@
       <c r="E117" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F117" s="17" t="n"/>
+      <c r="F117" s="18" t="n"/>
       <c r="G117" s="3">
         <f>IF(F117="","",F117-E117)</f>
         <v/>
@@ -6145,7 +6285,7 @@
       <c r="E118" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F118" s="17" t="n"/>
+      <c r="F118" s="18" t="n"/>
       <c r="G118" s="3">
         <f>IF(F118="","",F118-E118)</f>
         <v/>
@@ -6173,7 +6313,7 @@
       <c r="E119" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F119" s="17" t="n"/>
+      <c r="F119" s="18" t="n"/>
       <c r="G119" s="3">
         <f>IF(F119="","",F119-E119)</f>
         <v/>
@@ -6201,7 +6341,7 @@
       <c r="E120" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F120" s="17" t="n"/>
+      <c r="F120" s="18" t="n"/>
       <c r="G120" s="3">
         <f>IF(F120="","",F120-E120)</f>
         <v/>
@@ -6229,23 +6369,23 @@
       <c r="E121" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F121" s="17" t="n"/>
+      <c r="F121" s="18" t="n"/>
       <c r="G121" s="3">
         <f>IF(F121="","",F121-E121)</f>
         <v/>
       </c>
     </row>
     <row r="122">
-      <c r="D122" s="12" t="inlineStr">
+      <c r="D122" s="13" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E122" s="12">
+      <c r="E122" s="13">
         <f>SUM(E2:E121)</f>
         <v/>
       </c>
-      <c r="F122" s="12">
+      <c r="F122" s="13">
         <f>SUM(F2:F121)</f>
         <v/>
       </c>
@@ -6332,7 +6472,7 @@
       <c r="E2" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F2" s="17" t="n"/>
+      <c r="F2" s="18" t="n"/>
       <c r="G2" s="3">
         <f>IF(F2="","",F2-E2)</f>
         <v/>
@@ -6360,7 +6500,7 @@
       <c r="E3" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F3" s="17" t="n"/>
+      <c r="F3" s="18" t="n"/>
       <c r="G3" s="3">
         <f>IF(F3="","",F3-E3)</f>
         <v/>
@@ -6388,7 +6528,7 @@
       <c r="E4" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F4" s="17" t="n"/>
+      <c r="F4" s="18" t="n"/>
       <c r="G4" s="3">
         <f>IF(F4="","",F4-E4)</f>
         <v/>
@@ -6416,7 +6556,7 @@
       <c r="E5" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F5" s="17" t="n"/>
+      <c r="F5" s="18" t="n"/>
       <c r="G5" s="3">
         <f>IF(F5="","",F5-E5)</f>
         <v/>
@@ -6444,7 +6584,7 @@
       <c r="E6" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F6" s="17" t="n"/>
+      <c r="F6" s="18" t="n"/>
       <c r="G6" s="3">
         <f>IF(F6="","",F6-E6)</f>
         <v/>
@@ -6472,7 +6612,7 @@
       <c r="E7" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F7" s="17" t="n"/>
+      <c r="F7" s="18" t="n"/>
       <c r="G7" s="3">
         <f>IF(F7="","",F7-E7)</f>
         <v/>
@@ -6500,7 +6640,7 @@
       <c r="E8" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F8" s="17" t="n"/>
+      <c r="F8" s="18" t="n"/>
       <c r="G8" s="3">
         <f>IF(F8="","",F8-E8)</f>
         <v/>
@@ -6528,7 +6668,7 @@
       <c r="E9" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F9" s="17" t="n"/>
+      <c r="F9" s="18" t="n"/>
       <c r="G9" s="3">
         <f>IF(F9="","",F9-E9)</f>
         <v/>
@@ -6556,7 +6696,7 @@
       <c r="E10" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F10" s="17" t="n"/>
+      <c r="F10" s="18" t="n"/>
       <c r="G10" s="3">
         <f>IF(F10="","",F10-E10)</f>
         <v/>
@@ -6584,7 +6724,7 @@
       <c r="E11" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F11" s="17" t="n"/>
+      <c r="F11" s="18" t="n"/>
       <c r="G11" s="3">
         <f>IF(F11="","",F11-E11)</f>
         <v/>
@@ -6612,7 +6752,7 @@
       <c r="E12" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F12" s="17" t="n"/>
+      <c r="F12" s="18" t="n"/>
       <c r="G12" s="3">
         <f>IF(F12="","",F12-E12)</f>
         <v/>
@@ -6640,7 +6780,7 @@
       <c r="E13" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F13" s="17" t="n"/>
+      <c r="F13" s="18" t="n"/>
       <c r="G13" s="3">
         <f>IF(F13="","",F13-E13)</f>
         <v/>
@@ -6668,7 +6808,7 @@
       <c r="E14" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F14" s="17" t="n"/>
+      <c r="F14" s="18" t="n"/>
       <c r="G14" s="3">
         <f>IF(F14="","",F14-E14)</f>
         <v/>
@@ -6696,7 +6836,7 @@
       <c r="E15" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F15" s="17" t="n"/>
+      <c r="F15" s="18" t="n"/>
       <c r="G15" s="3">
         <f>IF(F15="","",F15-E15)</f>
         <v/>
@@ -6724,7 +6864,7 @@
       <c r="E16" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F16" s="17" t="n"/>
+      <c r="F16" s="18" t="n"/>
       <c r="G16" s="3">
         <f>IF(F16="","",F16-E16)</f>
         <v/>
@@ -6752,7 +6892,7 @@
       <c r="E17" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F17" s="17" t="n"/>
+      <c r="F17" s="18" t="n"/>
       <c r="G17" s="3">
         <f>IF(F17="","",F17-E17)</f>
         <v/>
@@ -6780,7 +6920,7 @@
       <c r="E18" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F18" s="17" t="n"/>
+      <c r="F18" s="18" t="n"/>
       <c r="G18" s="3">
         <f>IF(F18="","",F18-E18)</f>
         <v/>
@@ -6808,7 +6948,7 @@
       <c r="E19" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F19" s="17" t="n"/>
+      <c r="F19" s="18" t="n"/>
       <c r="G19" s="3">
         <f>IF(F19="","",F19-E19)</f>
         <v/>
@@ -6836,7 +6976,7 @@
       <c r="E20" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F20" s="17" t="n"/>
+      <c r="F20" s="18" t="n"/>
       <c r="G20" s="3">
         <f>IF(F20="","",F20-E20)</f>
         <v/>
@@ -6864,7 +7004,7 @@
       <c r="E21" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F21" s="17" t="n"/>
+      <c r="F21" s="18" t="n"/>
       <c r="G21" s="3">
         <f>IF(F21="","",F21-E21)</f>
         <v/>
@@ -6892,7 +7032,7 @@
       <c r="E22" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F22" s="17" t="n"/>
+      <c r="F22" s="18" t="n"/>
       <c r="G22" s="3">
         <f>IF(F22="","",F22-E22)</f>
         <v/>
@@ -6920,7 +7060,7 @@
       <c r="E23" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F23" s="17" t="n"/>
+      <c r="F23" s="18" t="n"/>
       <c r="G23" s="3">
         <f>IF(F23="","",F23-E23)</f>
         <v/>
@@ -6948,7 +7088,7 @@
       <c r="E24" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F24" s="17" t="n"/>
+      <c r="F24" s="18" t="n"/>
       <c r="G24" s="3">
         <f>IF(F24="","",F24-E24)</f>
         <v/>
@@ -6976,7 +7116,7 @@
       <c r="E25" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F25" s="17" t="n"/>
+      <c r="F25" s="18" t="n"/>
       <c r="G25" s="3">
         <f>IF(F25="","",F25-E25)</f>
         <v/>
@@ -7004,7 +7144,7 @@
       <c r="E26" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F26" s="17" t="n"/>
+      <c r="F26" s="18" t="n"/>
       <c r="G26" s="3">
         <f>IF(F26="","",F26-E26)</f>
         <v/>
@@ -7032,7 +7172,7 @@
       <c r="E27" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F27" s="17" t="n"/>
+      <c r="F27" s="18" t="n"/>
       <c r="G27" s="3">
         <f>IF(F27="","",F27-E27)</f>
         <v/>
@@ -7060,7 +7200,7 @@
       <c r="E28" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F28" s="17" t="n"/>
+      <c r="F28" s="18" t="n"/>
       <c r="G28" s="3">
         <f>IF(F28="","",F28-E28)</f>
         <v/>
@@ -7088,7 +7228,7 @@
       <c r="E29" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F29" s="17" t="n"/>
+      <c r="F29" s="18" t="n"/>
       <c r="G29" s="3">
         <f>IF(F29="","",F29-E29)</f>
         <v/>
@@ -7116,7 +7256,7 @@
       <c r="E30" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F30" s="17" t="n"/>
+      <c r="F30" s="18" t="n"/>
       <c r="G30" s="3">
         <f>IF(F30="","",F30-E30)</f>
         <v/>
@@ -7144,7 +7284,7 @@
       <c r="E31" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F31" s="17" t="n"/>
+      <c r="F31" s="18" t="n"/>
       <c r="G31" s="3">
         <f>IF(F31="","",F31-E31)</f>
         <v/>
@@ -7172,7 +7312,7 @@
       <c r="E32" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F32" s="17" t="n"/>
+      <c r="F32" s="18" t="n"/>
       <c r="G32" s="3">
         <f>IF(F32="","",F32-E32)</f>
         <v/>
@@ -7200,7 +7340,7 @@
       <c r="E33" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F33" s="17" t="n"/>
+      <c r="F33" s="18" t="n"/>
       <c r="G33" s="3">
         <f>IF(F33="","",F33-E33)</f>
         <v/>
@@ -7228,7 +7368,7 @@
       <c r="E34" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F34" s="17" t="n"/>
+      <c r="F34" s="18" t="n"/>
       <c r="G34" s="3">
         <f>IF(F34="","",F34-E34)</f>
         <v/>
@@ -7256,7 +7396,7 @@
       <c r="E35" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F35" s="17" t="n"/>
+      <c r="F35" s="18" t="n"/>
       <c r="G35" s="3">
         <f>IF(F35="","",F35-E35)</f>
         <v/>
@@ -7284,7 +7424,7 @@
       <c r="E36" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F36" s="17" t="n"/>
+      <c r="F36" s="18" t="n"/>
       <c r="G36" s="3">
         <f>IF(F36="","",F36-E36)</f>
         <v/>
@@ -7312,7 +7452,7 @@
       <c r="E37" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F37" s="17" t="n"/>
+      <c r="F37" s="18" t="n"/>
       <c r="G37" s="3">
         <f>IF(F37="","",F37-E37)</f>
         <v/>
@@ -7340,7 +7480,7 @@
       <c r="E38" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F38" s="17" t="n"/>
+      <c r="F38" s="18" t="n"/>
       <c r="G38" s="3">
         <f>IF(F38="","",F38-E38)</f>
         <v/>
@@ -7368,7 +7508,7 @@
       <c r="E39" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F39" s="17" t="n"/>
+      <c r="F39" s="18" t="n"/>
       <c r="G39" s="3">
         <f>IF(F39="","",F39-E39)</f>
         <v/>
@@ -7396,7 +7536,7 @@
       <c r="E40" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F40" s="17" t="n"/>
+      <c r="F40" s="18" t="n"/>
       <c r="G40" s="3">
         <f>IF(F40="","",F40-E40)</f>
         <v/>
@@ -7424,7 +7564,7 @@
       <c r="E41" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F41" s="17" t="n"/>
+      <c r="F41" s="18" t="n"/>
       <c r="G41" s="3">
         <f>IF(F41="","",F41-E41)</f>
         <v/>
@@ -7452,7 +7592,7 @@
       <c r="E42" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F42" s="17" t="n"/>
+      <c r="F42" s="18" t="n"/>
       <c r="G42" s="3">
         <f>IF(F42="","",F42-E42)</f>
         <v/>
@@ -7480,7 +7620,7 @@
       <c r="E43" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F43" s="17" t="n"/>
+      <c r="F43" s="18" t="n"/>
       <c r="G43" s="3">
         <f>IF(F43="","",F43-E43)</f>
         <v/>
@@ -7508,7 +7648,7 @@
       <c r="E44" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F44" s="17" t="n"/>
+      <c r="F44" s="18" t="n"/>
       <c r="G44" s="3">
         <f>IF(F44="","",F44-E44)</f>
         <v/>
@@ -7536,7 +7676,7 @@
       <c r="E45" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F45" s="17" t="n"/>
+      <c r="F45" s="18" t="n"/>
       <c r="G45" s="3">
         <f>IF(F45="","",F45-E45)</f>
         <v/>
@@ -7564,7 +7704,7 @@
       <c r="E46" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F46" s="17" t="n"/>
+      <c r="F46" s="18" t="n"/>
       <c r="G46" s="3">
         <f>IF(F46="","",F46-E46)</f>
         <v/>
@@ -7592,7 +7732,7 @@
       <c r="E47" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F47" s="17" t="n"/>
+      <c r="F47" s="18" t="n"/>
       <c r="G47" s="3">
         <f>IF(F47="","",F47-E47)</f>
         <v/>
@@ -7620,7 +7760,7 @@
       <c r="E48" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F48" s="17" t="n"/>
+      <c r="F48" s="18" t="n"/>
       <c r="G48" s="3">
         <f>IF(F48="","",F48-E48)</f>
         <v/>
@@ -7648,7 +7788,7 @@
       <c r="E49" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F49" s="17" t="n"/>
+      <c r="F49" s="18" t="n"/>
       <c r="G49" s="3">
         <f>IF(F49="","",F49-E49)</f>
         <v/>
@@ -7676,7 +7816,7 @@
       <c r="E50" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F50" s="17" t="n"/>
+      <c r="F50" s="18" t="n"/>
       <c r="G50" s="3">
         <f>IF(F50="","",F50-E50)</f>
         <v/>
@@ -7704,7 +7844,7 @@
       <c r="E51" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F51" s="17" t="n"/>
+      <c r="F51" s="18" t="n"/>
       <c r="G51" s="3">
         <f>IF(F51="","",F51-E51)</f>
         <v/>
@@ -7732,7 +7872,7 @@
       <c r="E52" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F52" s="17" t="n"/>
+      <c r="F52" s="18" t="n"/>
       <c r="G52" s="3">
         <f>IF(F52="","",F52-E52)</f>
         <v/>
@@ -7760,7 +7900,7 @@
       <c r="E53" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F53" s="17" t="n"/>
+      <c r="F53" s="18" t="n"/>
       <c r="G53" s="3">
         <f>IF(F53="","",F53-E53)</f>
         <v/>
@@ -7788,7 +7928,7 @@
       <c r="E54" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F54" s="17" t="n"/>
+      <c r="F54" s="18" t="n"/>
       <c r="G54" s="3">
         <f>IF(F54="","",F54-E54)</f>
         <v/>
@@ -7816,7 +7956,7 @@
       <c r="E55" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F55" s="17" t="n"/>
+      <c r="F55" s="18" t="n"/>
       <c r="G55" s="3">
         <f>IF(F55="","",F55-E55)</f>
         <v/>
@@ -7844,7 +7984,7 @@
       <c r="E56" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F56" s="17" t="n"/>
+      <c r="F56" s="18" t="n"/>
       <c r="G56" s="3">
         <f>IF(F56="","",F56-E56)</f>
         <v/>
@@ -7872,7 +8012,7 @@
       <c r="E57" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F57" s="17" t="n"/>
+      <c r="F57" s="18" t="n"/>
       <c r="G57" s="3">
         <f>IF(F57="","",F57-E57)</f>
         <v/>
@@ -7900,7 +8040,7 @@
       <c r="E58" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F58" s="17" t="n"/>
+      <c r="F58" s="18" t="n"/>
       <c r="G58" s="3">
         <f>IF(F58="","",F58-E58)</f>
         <v/>
@@ -7928,7 +8068,7 @@
       <c r="E59" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F59" s="17" t="n"/>
+      <c r="F59" s="18" t="n"/>
       <c r="G59" s="3">
         <f>IF(F59="","",F59-E59)</f>
         <v/>
@@ -7956,7 +8096,7 @@
       <c r="E60" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F60" s="17" t="n"/>
+      <c r="F60" s="18" t="n"/>
       <c r="G60" s="3">
         <f>IF(F60="","",F60-E60)</f>
         <v/>
@@ -7984,7 +8124,7 @@
       <c r="E61" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F61" s="17" t="n"/>
+      <c r="F61" s="18" t="n"/>
       <c r="G61" s="3">
         <f>IF(F61="","",F61-E61)</f>
         <v/>
@@ -8012,7 +8152,7 @@
       <c r="E62" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F62" s="17" t="n"/>
+      <c r="F62" s="18" t="n"/>
       <c r="G62" s="3">
         <f>IF(F62="","",F62-E62)</f>
         <v/>
@@ -8040,7 +8180,7 @@
       <c r="E63" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F63" s="17" t="n"/>
+      <c r="F63" s="18" t="n"/>
       <c r="G63" s="3">
         <f>IF(F63="","",F63-E63)</f>
         <v/>
@@ -8068,7 +8208,7 @@
       <c r="E64" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F64" s="17" t="n"/>
+      <c r="F64" s="18" t="n"/>
       <c r="G64" s="3">
         <f>IF(F64="","",F64-E64)</f>
         <v/>
@@ -8096,7 +8236,7 @@
       <c r="E65" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F65" s="17" t="n"/>
+      <c r="F65" s="18" t="n"/>
       <c r="G65" s="3">
         <f>IF(F65="","",F65-E65)</f>
         <v/>
@@ -8124,7 +8264,7 @@
       <c r="E66" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F66" s="17" t="n"/>
+      <c r="F66" s="18" t="n"/>
       <c r="G66" s="3">
         <f>IF(F66="","",F66-E66)</f>
         <v/>
@@ -8152,7 +8292,7 @@
       <c r="E67" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F67" s="17" t="n"/>
+      <c r="F67" s="18" t="n"/>
       <c r="G67" s="3">
         <f>IF(F67="","",F67-E67)</f>
         <v/>
@@ -8180,7 +8320,7 @@
       <c r="E68" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F68" s="17" t="n"/>
+      <c r="F68" s="18" t="n"/>
       <c r="G68" s="3">
         <f>IF(F68="","",F68-E68)</f>
         <v/>
@@ -8208,7 +8348,7 @@
       <c r="E69" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F69" s="17" t="n"/>
+      <c r="F69" s="18" t="n"/>
       <c r="G69" s="3">
         <f>IF(F69="","",F69-E69)</f>
         <v/>
@@ -8236,7 +8376,7 @@
       <c r="E70" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F70" s="17" t="n"/>
+      <c r="F70" s="18" t="n"/>
       <c r="G70" s="3">
         <f>IF(F70="","",F70-E70)</f>
         <v/>
@@ -8264,7 +8404,7 @@
       <c r="E71" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F71" s="17" t="n"/>
+      <c r="F71" s="18" t="n"/>
       <c r="G71" s="3">
         <f>IF(F71="","",F71-E71)</f>
         <v/>
@@ -8292,7 +8432,7 @@
       <c r="E72" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F72" s="17" t="n"/>
+      <c r="F72" s="18" t="n"/>
       <c r="G72" s="3">
         <f>IF(F72="","",F72-E72)</f>
         <v/>
@@ -8320,7 +8460,7 @@
       <c r="E73" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F73" s="17" t="n"/>
+      <c r="F73" s="18" t="n"/>
       <c r="G73" s="3">
         <f>IF(F73="","",F73-E73)</f>
         <v/>
@@ -8348,7 +8488,7 @@
       <c r="E74" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F74" s="17" t="n"/>
+      <c r="F74" s="18" t="n"/>
       <c r="G74" s="3">
         <f>IF(F74="","",F74-E74)</f>
         <v/>
@@ -8376,7 +8516,7 @@
       <c r="E75" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F75" s="17" t="n"/>
+      <c r="F75" s="18" t="n"/>
       <c r="G75" s="3">
         <f>IF(F75="","",F75-E75)</f>
         <v/>
@@ -8404,7 +8544,7 @@
       <c r="E76" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F76" s="17" t="n"/>
+      <c r="F76" s="18" t="n"/>
       <c r="G76" s="3">
         <f>IF(F76="","",F76-E76)</f>
         <v/>
@@ -8432,7 +8572,7 @@
       <c r="E77" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F77" s="17" t="n"/>
+      <c r="F77" s="18" t="n"/>
       <c r="G77" s="3">
         <f>IF(F77="","",F77-E77)</f>
         <v/>
@@ -8460,7 +8600,7 @@
       <c r="E78" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F78" s="17" t="n"/>
+      <c r="F78" s="18" t="n"/>
       <c r="G78" s="3">
         <f>IF(F78="","",F78-E78)</f>
         <v/>
@@ -8488,7 +8628,7 @@
       <c r="E79" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F79" s="17" t="n"/>
+      <c r="F79" s="18" t="n"/>
       <c r="G79" s="3">
         <f>IF(F79="","",F79-E79)</f>
         <v/>
@@ -8516,7 +8656,7 @@
       <c r="E80" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F80" s="17" t="n"/>
+      <c r="F80" s="18" t="n"/>
       <c r="G80" s="3">
         <f>IF(F80="","",F80-E80)</f>
         <v/>
@@ -8544,7 +8684,7 @@
       <c r="E81" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F81" s="17" t="n"/>
+      <c r="F81" s="18" t="n"/>
       <c r="G81" s="3">
         <f>IF(F81="","",F81-E81)</f>
         <v/>
@@ -8572,7 +8712,7 @@
       <c r="E82" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F82" s="17" t="n"/>
+      <c r="F82" s="18" t="n"/>
       <c r="G82" s="3">
         <f>IF(F82="","",F82-E82)</f>
         <v/>
@@ -8600,7 +8740,7 @@
       <c r="E83" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F83" s="17" t="n"/>
+      <c r="F83" s="18" t="n"/>
       <c r="G83" s="3">
         <f>IF(F83="","",F83-E83)</f>
         <v/>
@@ -8628,7 +8768,7 @@
       <c r="E84" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F84" s="17" t="n"/>
+      <c r="F84" s="18" t="n"/>
       <c r="G84" s="3">
         <f>IF(F84="","",F84-E84)</f>
         <v/>
@@ -8656,7 +8796,7 @@
       <c r="E85" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F85" s="17" t="n"/>
+      <c r="F85" s="18" t="n"/>
       <c r="G85" s="3">
         <f>IF(F85="","",F85-E85)</f>
         <v/>
@@ -8684,7 +8824,7 @@
       <c r="E86" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F86" s="17" t="n"/>
+      <c r="F86" s="18" t="n"/>
       <c r="G86" s="3">
         <f>IF(F86="","",F86-E86)</f>
         <v/>
@@ -8712,7 +8852,7 @@
       <c r="E87" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F87" s="17" t="n"/>
+      <c r="F87" s="18" t="n"/>
       <c r="G87" s="3">
         <f>IF(F87="","",F87-E87)</f>
         <v/>
@@ -8740,7 +8880,7 @@
       <c r="E88" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F88" s="17" t="n"/>
+      <c r="F88" s="18" t="n"/>
       <c r="G88" s="3">
         <f>IF(F88="","",F88-E88)</f>
         <v/>
@@ -8768,7 +8908,7 @@
       <c r="E89" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F89" s="17" t="n"/>
+      <c r="F89" s="18" t="n"/>
       <c r="G89" s="3">
         <f>IF(F89="","",F89-E89)</f>
         <v/>
@@ -8796,7 +8936,7 @@
       <c r="E90" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F90" s="17" t="n"/>
+      <c r="F90" s="18" t="n"/>
       <c r="G90" s="3">
         <f>IF(F90="","",F90-E90)</f>
         <v/>
@@ -8824,7 +8964,7 @@
       <c r="E91" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F91" s="17" t="n"/>
+      <c r="F91" s="18" t="n"/>
       <c r="G91" s="3">
         <f>IF(F91="","",F91-E91)</f>
         <v/>
@@ -8852,7 +8992,7 @@
       <c r="E92" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F92" s="17" t="n"/>
+      <c r="F92" s="18" t="n"/>
       <c r="G92" s="3">
         <f>IF(F92="","",F92-E92)</f>
         <v/>
@@ -8880,7 +9020,7 @@
       <c r="E93" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F93" s="17" t="n"/>
+      <c r="F93" s="18" t="n"/>
       <c r="G93" s="3">
         <f>IF(F93="","",F93-E93)</f>
         <v/>
@@ -8908,7 +9048,7 @@
       <c r="E94" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F94" s="17" t="n"/>
+      <c r="F94" s="18" t="n"/>
       <c r="G94" s="3">
         <f>IF(F94="","",F94-E94)</f>
         <v/>
@@ -8936,7 +9076,7 @@
       <c r="E95" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F95" s="17" t="n"/>
+      <c r="F95" s="18" t="n"/>
       <c r="G95" s="3">
         <f>IF(F95="","",F95-E95)</f>
         <v/>
@@ -8964,7 +9104,7 @@
       <c r="E96" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F96" s="17" t="n"/>
+      <c r="F96" s="18" t="n"/>
       <c r="G96" s="3">
         <f>IF(F96="","",F96-E96)</f>
         <v/>
@@ -8992,7 +9132,7 @@
       <c r="E97" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F97" s="17" t="n"/>
+      <c r="F97" s="18" t="n"/>
       <c r="G97" s="3">
         <f>IF(F97="","",F97-E97)</f>
         <v/>
@@ -9020,7 +9160,7 @@
       <c r="E98" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F98" s="17" t="n"/>
+      <c r="F98" s="18" t="n"/>
       <c r="G98" s="3">
         <f>IF(F98="","",F98-E98)</f>
         <v/>
@@ -9048,7 +9188,7 @@
       <c r="E99" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F99" s="17" t="n"/>
+      <c r="F99" s="18" t="n"/>
       <c r="G99" s="3">
         <f>IF(F99="","",F99-E99)</f>
         <v/>
@@ -9076,7 +9216,7 @@
       <c r="E100" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F100" s="17" t="n"/>
+      <c r="F100" s="18" t="n"/>
       <c r="G100" s="3">
         <f>IF(F100="","",F100-E100)</f>
         <v/>
@@ -9104,7 +9244,7 @@
       <c r="E101" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F101" s="17" t="n"/>
+      <c r="F101" s="18" t="n"/>
       <c r="G101" s="3">
         <f>IF(F101="","",F101-E101)</f>
         <v/>
@@ -9132,7 +9272,7 @@
       <c r="E102" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F102" s="17" t="n"/>
+      <c r="F102" s="18" t="n"/>
       <c r="G102" s="3">
         <f>IF(F102="","",F102-E102)</f>
         <v/>
@@ -9160,7 +9300,7 @@
       <c r="E103" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F103" s="17" t="n"/>
+      <c r="F103" s="18" t="n"/>
       <c r="G103" s="3">
         <f>IF(F103="","",F103-E103)</f>
         <v/>
@@ -9188,7 +9328,7 @@
       <c r="E104" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F104" s="17" t="n"/>
+      <c r="F104" s="18" t="n"/>
       <c r="G104" s="3">
         <f>IF(F104="","",F104-E104)</f>
         <v/>
@@ -9216,7 +9356,7 @@
       <c r="E105" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F105" s="17" t="n"/>
+      <c r="F105" s="18" t="n"/>
       <c r="G105" s="3">
         <f>IF(F105="","",F105-E105)</f>
         <v/>
@@ -9244,7 +9384,7 @@
       <c r="E106" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F106" s="17" t="n"/>
+      <c r="F106" s="18" t="n"/>
       <c r="G106" s="3">
         <f>IF(F106="","",F106-E106)</f>
         <v/>
@@ -9272,7 +9412,7 @@
       <c r="E107" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F107" s="17" t="n"/>
+      <c r="F107" s="18" t="n"/>
       <c r="G107" s="3">
         <f>IF(F107="","",F107-E107)</f>
         <v/>
@@ -9300,7 +9440,7 @@
       <c r="E108" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F108" s="17" t="n"/>
+      <c r="F108" s="18" t="n"/>
       <c r="G108" s="3">
         <f>IF(F108="","",F108-E108)</f>
         <v/>
@@ -9328,7 +9468,7 @@
       <c r="E109" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F109" s="17" t="n"/>
+      <c r="F109" s="18" t="n"/>
       <c r="G109" s="3">
         <f>IF(F109="","",F109-E109)</f>
         <v/>
@@ -9356,7 +9496,7 @@
       <c r="E110" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F110" s="17" t="n"/>
+      <c r="F110" s="18" t="n"/>
       <c r="G110" s="3">
         <f>IF(F110="","",F110-E110)</f>
         <v/>
@@ -9384,7 +9524,7 @@
       <c r="E111" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F111" s="17" t="n"/>
+      <c r="F111" s="18" t="n"/>
       <c r="G111" s="3">
         <f>IF(F111="","",F111-E111)</f>
         <v/>
@@ -9412,7 +9552,7 @@
       <c r="E112" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F112" s="17" t="n"/>
+      <c r="F112" s="18" t="n"/>
       <c r="G112" s="3">
         <f>IF(F112="","",F112-E112)</f>
         <v/>
@@ -9440,7 +9580,7 @@
       <c r="E113" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F113" s="17" t="n"/>
+      <c r="F113" s="18" t="n"/>
       <c r="G113" s="3">
         <f>IF(F113="","",F113-E113)</f>
         <v/>
@@ -9468,7 +9608,7 @@
       <c r="E114" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F114" s="17" t="n"/>
+      <c r="F114" s="18" t="n"/>
       <c r="G114" s="3">
         <f>IF(F114="","",F114-E114)</f>
         <v/>
@@ -9496,7 +9636,7 @@
       <c r="E115" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F115" s="17" t="n"/>
+      <c r="F115" s="18" t="n"/>
       <c r="G115" s="3">
         <f>IF(F115="","",F115-E115)</f>
         <v/>
@@ -9524,23 +9664,23 @@
       <c r="E116" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F116" s="17" t="n"/>
+      <c r="F116" s="18" t="n"/>
       <c r="G116" s="3">
         <f>IF(F116="","",F116-E116)</f>
         <v/>
       </c>
     </row>
     <row r="117">
-      <c r="D117" s="12" t="inlineStr">
+      <c r="D117" s="13" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E117" s="12">
+      <c r="E117" s="13">
         <f>SUM(E2:E116)</f>
         <v/>
       </c>
-      <c r="F117" s="12">
+      <c r="F117" s="13">
         <f>SUM(F2:F116)</f>
         <v/>
       </c>
@@ -9635,11 +9775,11 @@
           <t>Taux d'abandon</t>
         </is>
       </c>
-      <c r="B5" s="18">
+      <c r="B5" s="19">
         <f>IF(B3="","",B4/B3)</f>
         <v/>
       </c>
-      <c r="C5" s="18">
+      <c r="C5" s="19">
         <f>IF(C3="","",C4/C3)</f>
         <v/>
       </c>
@@ -9683,11 +9823,11 @@
           <t>Taux de réussite</t>
         </is>
       </c>
-      <c r="B8" s="18">
+      <c r="B8" s="19">
         <f>IF(B6="","",B7/B6)</f>
         <v/>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="19">
         <f>IF(C6="","",C7/C6)</f>
         <v/>
       </c>
@@ -9731,11 +9871,11 @@
           <t>Taux d'insertion à 6 mois</t>
         </is>
       </c>
-      <c r="B11" s="18">
+      <c r="B11" s="19">
         <f>IF(B3="","",B10/(B3-B4))</f>
         <v/>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="19">
         <f>IF(C3="","",C10/(C3-C4))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Livrets d'accueil MEM et RPMS, fiche lieu, étude tarifaire et déclinaisons du logo
- Livrets d'accueil au format du livret Marilyn (HTML imprimé par Chromium) :
  A5 lecture écran et A4 paysage imposé en livret plié, sommaire paginé,
  année en un coup d'œil, calendrier mensuel, accès en bus, restauration,
  règlement intérieur YEBA-DOC-04 et avenant.
- LIEU-01 : fiche « Votre lieu de formation » (Secrétariat Center, Technor).
- TAR-01 : concurrents, plafonds des financeurs, trois scénarios par titre ;
  feuille « Scénarios tarifaires » dans le classeur.
- Logo PNG décliné : fond clair (FORMATIONS en bleu), fond bleu, carrés,
  icônes ; polices Montserrat et Inter embarquées.
- Effectif de 10 stagiaires par promotion.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JZ6CWNerPeDJEuR1MPsUp5
</commit_message>
<xml_diff>
--- a/dossier-conformite-2026/livrables/05_Pilotage_annuel/PIL-03_Budget_tresorerie_tableau_de_bord.xlsx
+++ b/dossier-conformite-2026/livrables/05_Pilotage_annuel/PIL-03_Budget_tresorerie_tableau_de_bord.xlsx
@@ -12,8 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget RPMS" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heures MEM" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heures RPMS" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicateurs" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Absences" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scénarios tarifaires" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicateurs" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Absences" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,12 +23,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="#,##0 &quot;€&quot;"/>
     <numFmt numFmtId="167" formatCode="#,##0.00 &quot;€&quot;"/>
     <numFmt numFmtId="168" formatCode="mmmm yyyy"/>
+    <numFmt numFmtId="169" formatCode="0.00 &quot;€&quot;"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -120,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -164,6 +166,10 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -9696,6 +9702,300 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Titre</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Scénario</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Prix par stagiaire</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Heures en centre</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>€ / heure</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Stagiaires</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Chiffre d'affaires</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Location de salle</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Après salle</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>MEM</t>
+        </is>
+      </c>
+      <c r="B2" s="19" t="inlineStr">
+        <is>
+          <t>A — Accessible</t>
+        </is>
+      </c>
+      <c r="C2" s="20" t="n">
+        <v>4200</v>
+      </c>
+      <c r="D2" s="19" t="n">
+        <v>560</v>
+      </c>
+      <c r="E2" s="21">
+        <f>C2/D2</f>
+        <v/>
+      </c>
+      <c r="F2" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G2" s="20">
+        <f>C2*F2</f>
+        <v/>
+      </c>
+      <c r="H2" s="20">
+        <f>D2/7*100</f>
+        <v/>
+      </c>
+      <c r="I2" s="20">
+        <f>G2-H2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>MEM</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>B — Recommandé</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="n">
+        <v>4900</v>
+      </c>
+      <c r="D3" s="19" t="n">
+        <v>560</v>
+      </c>
+      <c r="E3" s="21">
+        <f>C3/D3</f>
+        <v/>
+      </c>
+      <c r="F3" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G3" s="20">
+        <f>C3*F3</f>
+        <v/>
+      </c>
+      <c r="H3" s="20">
+        <f>D3/7*100</f>
+        <v/>
+      </c>
+      <c r="I3" s="20">
+        <f>G3-H3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>MEM</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>C — Premium</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="n">
+        <v>5600</v>
+      </c>
+      <c r="D4" s="19" t="n">
+        <v>560</v>
+      </c>
+      <c r="E4" s="21">
+        <f>C4/D4</f>
+        <v/>
+      </c>
+      <c r="F4" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G4" s="20">
+        <f>C4*F4</f>
+        <v/>
+      </c>
+      <c r="H4" s="20">
+        <f>D4/7*100</f>
+        <v/>
+      </c>
+      <c r="I4" s="20">
+        <f>G4-H4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>RPMS</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>A — Accessible</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="n">
+        <v>4300</v>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>595</v>
+      </c>
+      <c r="E5" s="21">
+        <f>C5/D5</f>
+        <v/>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G5" s="20">
+        <f>C5*F5</f>
+        <v/>
+      </c>
+      <c r="H5" s="20">
+        <f>D5/7*100</f>
+        <v/>
+      </c>
+      <c r="I5" s="20">
+        <f>G5-H5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>RPMS</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>B — Recommandé</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="n">
+        <v>4950</v>
+      </c>
+      <c r="D6" s="19" t="n">
+        <v>595</v>
+      </c>
+      <c r="E6" s="21">
+        <f>C6/D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G6" s="20">
+        <f>C6*F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="20">
+        <f>D6/7*100</f>
+        <v/>
+      </c>
+      <c r="I6" s="20">
+        <f>G6-H6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>RPMS</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>C — Premium</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="n">
+        <v>5900</v>
+      </c>
+      <c r="D7" s="19" t="n">
+        <v>595</v>
+      </c>
+      <c r="E7" s="21">
+        <f>C7/D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G7" s="20">
+        <f>C7*F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="20">
+        <f>D7/7*100</f>
+        <v/>
+      </c>
+      <c r="I7" s="20">
+        <f>G7-H7</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -9775,11 +10075,11 @@
           <t>Taux d'abandon</t>
         </is>
       </c>
-      <c r="B5" s="19">
+      <c r="B5" s="23">
         <f>IF(B3="","",B4/B3)</f>
         <v/>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="23">
         <f>IF(C3="","",C4/C3)</f>
         <v/>
       </c>
@@ -9823,11 +10123,11 @@
           <t>Taux de réussite</t>
         </is>
       </c>
-      <c r="B8" s="19">
+      <c r="B8" s="23">
         <f>IF(B6="","",B7/B6)</f>
         <v/>
       </c>
-      <c r="C8" s="19">
+      <c r="C8" s="23">
         <f>IF(C6="","",C7/C6)</f>
         <v/>
       </c>
@@ -9871,11 +10171,11 @@
           <t>Taux d'insertion à 6 mois</t>
         </is>
       </c>
-      <c r="B11" s="19">
+      <c r="B11" s="23">
         <f>IF(B3="","",B10/(B3-B4))</f>
         <v/>
       </c>
-      <c r="C11" s="19">
+      <c r="C11" s="23">
         <f>IF(C3="","",C10/(C3-C4))</f>
         <v/>
       </c>
@@ -9890,7 +10190,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>